<commit_message>
feat: abas de notas bimestrais com formatação condicional
</commit_message>
<xml_diff>
--- a/diario-de-classe.xlsx
+++ b/diario-de-classe.xlsx
@@ -18,6 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presença - Set" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presença - Out" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presença - Nov" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B1" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B2" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B3" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B4" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,8 +30,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,15 +90,32 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4435,6 +4457,2398 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Média Geral</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <f>Turma!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="4">
+        <f>IFERROR(AVERAGE(C2:H2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Turma!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="4">
+        <f>IFERROR(AVERAGE(C3:H3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Turma!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="4">
+        <f>IFERROR(AVERAGE(C4:H4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Turma!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="4">
+        <f>IFERROR(AVERAGE(C5:H5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Turma!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="4">
+        <f>IFERROR(AVERAGE(C6:H6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Turma!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="4">
+        <f>IFERROR(AVERAGE(C7:H7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Turma!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="4">
+        <f>IFERROR(AVERAGE(C8:H8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Turma!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="4">
+        <f>IFERROR(AVERAGE(C9:H9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Turma!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="4">
+        <f>IFERROR(AVERAGE(C10:H10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <f>Turma!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="4">
+        <f>IFERROR(AVERAGE(C11:H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <f>Turma!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="4">
+        <f>IFERROR(AVERAGE(C12:H12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>Turma!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="4">
+        <f>IFERROR(AVERAGE(C13:H13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <f>Turma!B14</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="4">
+        <f>IFERROR(AVERAGE(C14:H14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <f>Turma!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="4">
+        <f>IFERROR(AVERAGE(C15:H15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <f>Turma!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="4">
+        <f>IFERROR(AVERAGE(C16:H16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2">
+        <f>Turma!B17</f>
+        <v/>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="4">
+        <f>IFERROR(AVERAGE(C17:H17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2">
+        <f>Turma!B18</f>
+        <v/>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="4">
+        <f>IFERROR(AVERAGE(C18:H18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2">
+        <f>Turma!B19</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="4">
+        <f>IFERROR(AVERAGE(C19:H19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
+        <f>Turma!B20</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="4">
+        <f>IFERROR(AVERAGE(C20:H20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
+        <f>Turma!B21</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="4">
+        <f>IFERROR(AVERAGE(C21:H21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2">
+        <f>Turma!B22</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="4">
+        <f>IFERROR(AVERAGE(C22:H22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2">
+        <f>Turma!B23</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="4">
+        <f>IFERROR(AVERAGE(C23:H23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <f>Turma!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="4">
+        <f>IFERROR(AVERAGE(C24:H24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2">
+        <f>Turma!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="4">
+        <f>IFERROR(AVERAGE(C25:H25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2">
+        <f>Turma!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="4">
+        <f>IFERROR(AVERAGE(C26:H26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <f>Turma!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="4">
+        <f>IFERROR(AVERAGE(C27:H27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2">
+        <f>Turma!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="4">
+        <f>IFERROR(AVERAGE(C28:H28),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:I28">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>5</formula>
+      <formula>6.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Média Geral</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <f>Turma!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="4">
+        <f>IFERROR(AVERAGE(C2:H2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Turma!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="4">
+        <f>IFERROR(AVERAGE(C3:H3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Turma!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="4">
+        <f>IFERROR(AVERAGE(C4:H4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Turma!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="4">
+        <f>IFERROR(AVERAGE(C5:H5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Turma!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="4">
+        <f>IFERROR(AVERAGE(C6:H6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Turma!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="4">
+        <f>IFERROR(AVERAGE(C7:H7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Turma!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="4">
+        <f>IFERROR(AVERAGE(C8:H8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Turma!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="4">
+        <f>IFERROR(AVERAGE(C9:H9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Turma!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="4">
+        <f>IFERROR(AVERAGE(C10:H10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <f>Turma!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="4">
+        <f>IFERROR(AVERAGE(C11:H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <f>Turma!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="4">
+        <f>IFERROR(AVERAGE(C12:H12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>Turma!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="4">
+        <f>IFERROR(AVERAGE(C13:H13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <f>Turma!B14</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="4">
+        <f>IFERROR(AVERAGE(C14:H14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <f>Turma!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="4">
+        <f>IFERROR(AVERAGE(C15:H15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <f>Turma!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="4">
+        <f>IFERROR(AVERAGE(C16:H16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2">
+        <f>Turma!B17</f>
+        <v/>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="4">
+        <f>IFERROR(AVERAGE(C17:H17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2">
+        <f>Turma!B18</f>
+        <v/>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="4">
+        <f>IFERROR(AVERAGE(C18:H18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2">
+        <f>Turma!B19</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="4">
+        <f>IFERROR(AVERAGE(C19:H19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
+        <f>Turma!B20</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="4">
+        <f>IFERROR(AVERAGE(C20:H20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
+        <f>Turma!B21</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="4">
+        <f>IFERROR(AVERAGE(C21:H21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2">
+        <f>Turma!B22</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="4">
+        <f>IFERROR(AVERAGE(C22:H22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2">
+        <f>Turma!B23</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="4">
+        <f>IFERROR(AVERAGE(C23:H23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <f>Turma!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="4">
+        <f>IFERROR(AVERAGE(C24:H24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2">
+        <f>Turma!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="4">
+        <f>IFERROR(AVERAGE(C25:H25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2">
+        <f>Turma!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="4">
+        <f>IFERROR(AVERAGE(C26:H26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <f>Turma!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="4">
+        <f>IFERROR(AVERAGE(C27:H27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2">
+        <f>Turma!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="4">
+        <f>IFERROR(AVERAGE(C28:H28),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:I28">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>5</formula>
+      <formula>6.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Média Geral</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <f>Turma!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="4">
+        <f>IFERROR(AVERAGE(C2:H2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Turma!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="4">
+        <f>IFERROR(AVERAGE(C3:H3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Turma!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="4">
+        <f>IFERROR(AVERAGE(C4:H4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Turma!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="4">
+        <f>IFERROR(AVERAGE(C5:H5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Turma!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="4">
+        <f>IFERROR(AVERAGE(C6:H6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Turma!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="4">
+        <f>IFERROR(AVERAGE(C7:H7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Turma!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="4">
+        <f>IFERROR(AVERAGE(C8:H8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Turma!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="4">
+        <f>IFERROR(AVERAGE(C9:H9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Turma!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="4">
+        <f>IFERROR(AVERAGE(C10:H10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <f>Turma!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="4">
+        <f>IFERROR(AVERAGE(C11:H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <f>Turma!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="4">
+        <f>IFERROR(AVERAGE(C12:H12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>Turma!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="4">
+        <f>IFERROR(AVERAGE(C13:H13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <f>Turma!B14</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="4">
+        <f>IFERROR(AVERAGE(C14:H14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <f>Turma!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="4">
+        <f>IFERROR(AVERAGE(C15:H15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <f>Turma!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="4">
+        <f>IFERROR(AVERAGE(C16:H16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2">
+        <f>Turma!B17</f>
+        <v/>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="4">
+        <f>IFERROR(AVERAGE(C17:H17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2">
+        <f>Turma!B18</f>
+        <v/>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="4">
+        <f>IFERROR(AVERAGE(C18:H18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2">
+        <f>Turma!B19</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="4">
+        <f>IFERROR(AVERAGE(C19:H19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
+        <f>Turma!B20</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="4">
+        <f>IFERROR(AVERAGE(C20:H20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
+        <f>Turma!B21</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="4">
+        <f>IFERROR(AVERAGE(C21:H21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2">
+        <f>Turma!B22</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="4">
+        <f>IFERROR(AVERAGE(C22:H22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2">
+        <f>Turma!B23</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="4">
+        <f>IFERROR(AVERAGE(C23:H23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <f>Turma!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="4">
+        <f>IFERROR(AVERAGE(C24:H24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2">
+        <f>Turma!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="4">
+        <f>IFERROR(AVERAGE(C25:H25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2">
+        <f>Turma!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="4">
+        <f>IFERROR(AVERAGE(C26:H26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <f>Turma!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="4">
+        <f>IFERROR(AVERAGE(C27:H27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2">
+        <f>Turma!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="4">
+        <f>IFERROR(AVERAGE(C28:H28),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:I28">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>5</formula>
+      <formula>6.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Média Geral</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <f>Turma!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="4">
+        <f>IFERROR(AVERAGE(C2:H2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Turma!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="4">
+        <f>IFERROR(AVERAGE(C3:H3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Turma!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="4">
+        <f>IFERROR(AVERAGE(C4:H4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Turma!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="4">
+        <f>IFERROR(AVERAGE(C5:H5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Turma!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="4">
+        <f>IFERROR(AVERAGE(C6:H6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Turma!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="4">
+        <f>IFERROR(AVERAGE(C7:H7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Turma!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="4">
+        <f>IFERROR(AVERAGE(C8:H8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Turma!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="4">
+        <f>IFERROR(AVERAGE(C9:H9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Turma!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="4">
+        <f>IFERROR(AVERAGE(C10:H10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <f>Turma!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="4">
+        <f>IFERROR(AVERAGE(C11:H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <f>Turma!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="4">
+        <f>IFERROR(AVERAGE(C12:H12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>Turma!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="4">
+        <f>IFERROR(AVERAGE(C13:H13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <f>Turma!B14</f>
+        <v/>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="4">
+        <f>IFERROR(AVERAGE(C14:H14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <f>Turma!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="4">
+        <f>IFERROR(AVERAGE(C15:H15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <f>Turma!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="4">
+        <f>IFERROR(AVERAGE(C16:H16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2">
+        <f>Turma!B17</f>
+        <v/>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="4">
+        <f>IFERROR(AVERAGE(C17:H17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2">
+        <f>Turma!B18</f>
+        <v/>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="4">
+        <f>IFERROR(AVERAGE(C18:H18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2">
+        <f>Turma!B19</f>
+        <v/>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="4">
+        <f>IFERROR(AVERAGE(C19:H19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
+        <f>Turma!B20</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="4">
+        <f>IFERROR(AVERAGE(C20:H20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
+        <f>Turma!B21</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="4">
+        <f>IFERROR(AVERAGE(C21:H21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2">
+        <f>Turma!B22</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="4">
+        <f>IFERROR(AVERAGE(C22:H22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2">
+        <f>Turma!B23</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="4">
+        <f>IFERROR(AVERAGE(C23:H23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <f>Turma!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="4">
+        <f>IFERROR(AVERAGE(C24:H24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2">
+        <f>Turma!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="4">
+        <f>IFERROR(AVERAGE(C25:H25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2">
+        <f>Turma!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="4">
+        <f>IFERROR(AVERAGE(C26:H26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <f>Turma!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="4">
+        <f>IFERROR(AVERAGE(C27:H27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2">
+        <f>Turma!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="4">
+        <f>IFERROR(AVERAGE(C28:H28),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:I28">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>5</formula>
+      <formula>6.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: abas Recuperação, Contatos e Ocorrências
</commit_message>
<xml_diff>
--- a/diario-de-classe.xlsx
+++ b/diario-de-classe.xlsx
@@ -22,6 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B2" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B3" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas - B4" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuperação" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos e Reuniões" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocorrências" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +95,13 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6849,6 +6859,2265 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF0000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bimestre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nº Aluno</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nome do Aluno</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Disciplina</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Nota Original</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nota Recup.</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Situação Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2">
+        <f>IF(F2="","",IF(F2&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2">
+        <f>IF(F3="","",IF(F3&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2">
+        <f>IF(F4="","",IF(F4&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2">
+        <f>IF(F5="","",IF(F5&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2">
+        <f>IF(F6="","",IF(F6&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2">
+        <f>IF(F7="","",IF(F7&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2">
+        <f>IF(F8="","",IF(F8&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2">
+        <f>IF(F9="","",IF(F9&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2">
+        <f>IF(F10="","",IF(F10&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2">
+        <f>IF(F11="","",IF(F11&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2">
+        <f>IF(F12="","",IF(F12&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2">
+        <f>IF(F13="","",IF(F13&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2">
+        <f>IF(F14="","",IF(F14&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2">
+        <f>IF(F15="","",IF(F15&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2">
+        <f>IF(F16="","",IF(F16&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2">
+        <f>IF(F17="","",IF(F17&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2">
+        <f>IF(F18="","",IF(F18&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2">
+        <f>IF(F19="","",IF(F19&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2">
+        <f>IF(F20="","",IF(F20&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2">
+        <f>IF(F21="","",IF(F21&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2">
+        <f>IF(F22="","",IF(F22&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2">
+        <f>IF(F23="","",IF(F23&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2">
+        <f>IF(F24="","",IF(F24&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2">
+        <f>IF(F25="","",IF(F25&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2">
+        <f>IF(F26="","",IF(F26&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2">
+        <f>IF(F27="","",IF(F27&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2">
+        <f>IF(F28="","",IF(F28&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2">
+        <f>IF(F29="","",IF(F29&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2">
+        <f>IF(F30="","",IF(F30&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2">
+        <f>IF(F31="","",IF(F31&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2">
+        <f>IF(F32="","",IF(F32&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2">
+        <f>IF(F33="","",IF(F33&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2">
+        <f>IF(F34="","",IF(F34&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2">
+        <f>IF(F35="","",IF(F35&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2">
+        <f>IF(F36="","",IF(F36&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2">
+        <f>IF(F37="","",IF(F37&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2">
+        <f>IF(F38="","",IF(F38&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2">
+        <f>IF(F39="","",IF(F39&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2">
+        <f>IF(F40="","",IF(F40&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2">
+        <f>IF(F41="","",IF(F41&gt;=5,"Aprovado","Em recuperação"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2:G41">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Aprovado"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+      <formula>"Em recuperação"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF9900"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nº Aluno</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nome do Aluno</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Responsável</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Assunto</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Encaminhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="5" t="n"/>
+      <c r="G51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="5" t="n"/>
+      <c r="G52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="5" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="5" t="n"/>
+      <c r="G53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="5" t="n"/>
+      <c r="G58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="5" t="n"/>
+      <c r="G60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="5" t="n"/>
+      <c r="G62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="5" t="n"/>
+      <c r="G63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="5" t="n"/>
+      <c r="G64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="5" t="n"/>
+      <c r="G65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="5" t="n"/>
+      <c r="D67" s="5" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="5" t="n"/>
+      <c r="G67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="5" t="n"/>
+      <c r="D68" s="5" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="5" t="n"/>
+      <c r="G68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="5" t="n"/>
+      <c r="D69" s="5" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="5" t="n"/>
+      <c r="G69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="5" t="n"/>
+      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="5" t="n"/>
+      <c r="G70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="5" t="n"/>
+      <c r="D71" s="5" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="5" t="n"/>
+      <c r="G71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="5" t="n"/>
+      <c r="G72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="5" t="n"/>
+      <c r="D73" s="5" t="n"/>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="5" t="n"/>
+      <c r="G73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="2" t="n"/>
+      <c r="C75" s="5" t="n"/>
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="5" t="n"/>
+      <c r="G75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="5" t="n"/>
+      <c r="D76" s="5" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="5" t="n"/>
+      <c r="G76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="5" t="n"/>
+      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="5" t="n"/>
+      <c r="G77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="5" t="n"/>
+      <c r="G78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="5" t="n"/>
+      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="5" t="n"/>
+      <c r="G79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="5" t="n"/>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="5" t="n"/>
+      <c r="G80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="5" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="5" t="n"/>
+      <c r="G81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="5" t="n"/>
+      <c r="G82" s="5" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="5" t="n"/>
+      <c r="D83" s="5" t="n"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="5" t="n"/>
+      <c r="G83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="5" t="n"/>
+      <c r="D84" s="5" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="5" t="n"/>
+      <c r="G84" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="5" t="n"/>
+      <c r="D85" s="5" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="5" t="n"/>
+      <c r="G85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="5" t="n"/>
+      <c r="D86" s="5" t="n"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="5" t="n"/>
+      <c r="G86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="5" t="n"/>
+      <c r="D87" s="5" t="n"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="5" t="n"/>
+      <c r="G87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="5" t="n"/>
+      <c r="D88" s="5" t="n"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="5" t="n"/>
+      <c r="G88" s="5" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="5" t="n"/>
+      <c r="D89" s="5" t="n"/>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="5" t="n"/>
+      <c r="G89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="5" t="n"/>
+      <c r="D90" s="5" t="n"/>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="5" t="n"/>
+      <c r="G90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="5" t="n"/>
+      <c r="D91" s="5" t="n"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="5" t="n"/>
+      <c r="G91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="5" t="n"/>
+      <c r="D92" s="5" t="n"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="5" t="n"/>
+      <c r="G92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="5" t="n"/>
+      <c r="D93" s="5" t="n"/>
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="5" t="n"/>
+      <c r="G93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="5" t="n"/>
+      <c r="D94" s="5" t="n"/>
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="5" t="n"/>
+      <c r="G94" s="5" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="5" t="n"/>
+      <c r="D95" s="5" t="n"/>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="5" t="n"/>
+      <c r="D96" s="5" t="n"/>
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="5" t="n"/>
+      <c r="G96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="5" t="n"/>
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="5" t="n"/>
+      <c r="G97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="2" t="n"/>
+      <c r="C98" s="5" t="n"/>
+      <c r="D98" s="5" t="n"/>
+      <c r="E98" s="2" t="n"/>
+      <c r="F98" s="5" t="n"/>
+      <c r="G98" s="5" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="2" t="n"/>
+      <c r="C99" s="5" t="n"/>
+      <c r="D99" s="5" t="n"/>
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="5" t="n"/>
+      <c r="G99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n"/>
+      <c r="B100" s="2" t="n"/>
+      <c r="C100" s="5" t="n"/>
+      <c r="D100" s="5" t="n"/>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="5" t="n"/>
+      <c r="G100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n"/>
+      <c r="B101" s="2" t="n"/>
+      <c r="C101" s="5" t="n"/>
+      <c r="D101" s="5" t="n"/>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="5" t="n"/>
+      <c r="G101" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="009900FF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nº Aluno</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nome do Aluno</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Providência</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="6" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="6" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="6" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="6" t="n"/>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="6" t="n"/>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="6" t="n"/>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="6" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="6" t="n"/>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="6" t="n"/>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="7" t="n"/>
+      <c r="E44" s="7" t="n"/>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="6" t="n"/>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="7" t="n"/>
+      <c r="E45" s="7" t="n"/>
+    </row>
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="7" t="n"/>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="7" t="n"/>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="6" t="n"/>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="6" t="n"/>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="6" t="n"/>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="6" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="6" t="n"/>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="7" t="n"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="6" t="n"/>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="7" t="n"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="6" t="n"/>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="7" t="n"/>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="6" t="n"/>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="6" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="7" t="n"/>
+      <c r="E56" s="7" t="n"/>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="6" t="n"/>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="7" t="n"/>
+      <c r="E57" s="7" t="n"/>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="6" t="n"/>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="7" t="n"/>
+      <c r="E58" s="7" t="n"/>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="6" t="n"/>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="7" t="n"/>
+      <c r="E59" s="7" t="n"/>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="6" t="n"/>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="7" t="n"/>
+      <c r="E60" s="7" t="n"/>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="6" t="n"/>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="7" t="n"/>
+      <c r="D61" s="7" t="n"/>
+      <c r="E61" s="7" t="n"/>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="6" t="n"/>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="7" t="n"/>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="6" t="n"/>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="7" t="n"/>
+      <c r="D63" s="7" t="n"/>
+      <c r="E63" s="7" t="n"/>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="6" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="7" t="n"/>
+      <c r="E64" s="7" t="n"/>
+    </row>
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="6" t="n"/>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="7" t="n"/>
+      <c r="D65" s="7" t="n"/>
+      <c r="E65" s="7" t="n"/>
+    </row>
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="6" t="n"/>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="7" t="n"/>
+    </row>
+    <row r="67" ht="40" customHeight="1">
+      <c r="A67" s="6" t="n"/>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="7" t="n"/>
+    </row>
+    <row r="68" ht="40" customHeight="1">
+      <c r="A68" s="6" t="n"/>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="7" t="n"/>
+      <c r="D68" s="7" t="n"/>
+      <c r="E68" s="7" t="n"/>
+    </row>
+    <row r="69" ht="40" customHeight="1">
+      <c r="A69" s="6" t="n"/>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="7" t="n"/>
+    </row>
+    <row r="70" ht="40" customHeight="1">
+      <c r="A70" s="6" t="n"/>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="7" t="n"/>
+      <c r="D70" s="7" t="n"/>
+      <c r="E70" s="7" t="n"/>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="6" t="n"/>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="7" t="n"/>
+      <c r="D71" s="7" t="n"/>
+      <c r="E71" s="7" t="n"/>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="6" t="n"/>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="7" t="n"/>
+      <c r="D72" s="7" t="n"/>
+      <c r="E72" s="7" t="n"/>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="6" t="n"/>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="7" t="n"/>
+      <c r="D73" s="7" t="n"/>
+      <c r="E73" s="7" t="n"/>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="6" t="n"/>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="7" t="n"/>
+      <c r="D74" s="7" t="n"/>
+      <c r="E74" s="7" t="n"/>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="6" t="n"/>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="7" t="n"/>
+      <c r="E75" s="7" t="n"/>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="6" t="n"/>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="7" t="n"/>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="6" t="n"/>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="7" t="n"/>
+      <c r="D77" s="7" t="n"/>
+      <c r="E77" s="7" t="n"/>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="6" t="n"/>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="7" t="n"/>
+      <c r="D78" s="7" t="n"/>
+      <c r="E78" s="7" t="n"/>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="6" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="7" t="n"/>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="6" t="n"/>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="7" t="n"/>
+      <c r="D80" s="7" t="n"/>
+      <c r="E80" s="7" t="n"/>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="6" t="n"/>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="7" t="n"/>
+      <c r="D81" s="7" t="n"/>
+      <c r="E81" s="7" t="n"/>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="6" t="n"/>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="7" t="n"/>
+      <c r="D82" s="7" t="n"/>
+      <c r="E82" s="7" t="n"/>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="6" t="n"/>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="7" t="n"/>
+      <c r="D83" s="7" t="n"/>
+      <c r="E83" s="7" t="n"/>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="6" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="7" t="n"/>
+      <c r="D84" s="7" t="n"/>
+      <c r="E84" s="7" t="n"/>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="6" t="n"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="7" t="n"/>
+      <c r="D85" s="7" t="n"/>
+      <c r="E85" s="7" t="n"/>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="6" t="n"/>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="7" t="n"/>
+      <c r="D86" s="7" t="n"/>
+      <c r="E86" s="7" t="n"/>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="6" t="n"/>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="7" t="n"/>
+      <c r="D87" s="7" t="n"/>
+      <c r="E87" s="7" t="n"/>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="6" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="7" t="n"/>
+      <c r="D88" s="7" t="n"/>
+      <c r="E88" s="7" t="n"/>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="6" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="7" t="n"/>
+      <c r="D89" s="7" t="n"/>
+      <c r="E89" s="7" t="n"/>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="6" t="n"/>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="7" t="n"/>
+      <c r="D90" s="7" t="n"/>
+      <c r="E90" s="7" t="n"/>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="6" t="n"/>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="7" t="n"/>
+      <c r="D91" s="7" t="n"/>
+      <c r="E91" s="7" t="n"/>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="6" t="n"/>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="7" t="n"/>
+      <c r="D92" s="7" t="n"/>
+      <c r="E92" s="7" t="n"/>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="6" t="n"/>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="7" t="n"/>
+      <c r="D93" s="7" t="n"/>
+      <c r="E93" s="7" t="n"/>
+    </row>
+    <row r="94" ht="40" customHeight="1">
+      <c r="A94" s="6" t="n"/>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="7" t="n"/>
+      <c r="D94" s="7" t="n"/>
+      <c r="E94" s="7" t="n"/>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="A95" s="6" t="n"/>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="7" t="n"/>
+      <c r="D95" s="7" t="n"/>
+      <c r="E95" s="7" t="n"/>
+    </row>
+    <row r="96" ht="40" customHeight="1">
+      <c r="A96" s="6" t="n"/>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="7" t="n"/>
+      <c r="D96" s="7" t="n"/>
+      <c r="E96" s="7" t="n"/>
+    </row>
+    <row r="97" ht="40" customHeight="1">
+      <c r="A97" s="6" t="n"/>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="7" t="n"/>
+      <c r="D97" s="7" t="n"/>
+      <c r="E97" s="7" t="n"/>
+    </row>
+    <row r="98" ht="40" customHeight="1">
+      <c r="A98" s="6" t="n"/>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="7" t="n"/>
+      <c r="D98" s="7" t="n"/>
+      <c r="E98" s="7" t="n"/>
+    </row>
+    <row r="99" ht="40" customHeight="1">
+      <c r="A99" s="6" t="n"/>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="7" t="n"/>
+      <c r="D99" s="7" t="n"/>
+      <c r="E99" s="7" t="n"/>
+    </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="6" t="n"/>
+      <c r="B100" s="6" t="n"/>
+      <c r="C100" s="7" t="n"/>
+      <c r="D100" s="7" t="n"/>
+      <c r="E100" s="7" t="n"/>
+    </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="6" t="n"/>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="7" t="n"/>
+      <c r="D101" s="7" t="n"/>
+      <c r="E101" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: aba Resumo Anual com médias, frequência e situação final
</commit_message>
<xml_diff>
--- a/diario-de-classe.xlsx
+++ b/diario-de-classe.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recuperação" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos e Reuniões" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocorrências" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo Anual" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,7 +38,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +51,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +113,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9118,6 +9132,1099 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00404040"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>RESUMO ANUAL — 1º ANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Freq. %</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Média B1</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Média B2</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Média B3</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Média B4</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Média Final</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Turma!B3</f>
+        <v/>
+      </c>
+      <c r="C3" s="3">
+        <f>IFERROR(('Presença - Fev'!AK3+'Presença - Mar'!AK3+'Presença - Abr'!AK3+'Presença - Mai'!AK3+'Presença - Jun'!AK3+'Presença - Jul'!AK3+'Presença - Ago'!AK3+'Presença - Set'!AK3+'Presença - Out'!AK3+'Presença - Nov'!AK3)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>'Notas - B1'!I3</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>'Notas - B2'!I3</f>
+        <v/>
+      </c>
+      <c r="F3" s="4">
+        <f>'Notas - B3'!I3</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>'Notas - B4'!I3</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>IFERROR(AVERAGE(D3:G3),"")</f>
+        <v/>
+      </c>
+      <c r="I3" s="2">
+        <f>IF(H3="","",IF(AND(H3&gt;=5,C3&gt;=0.75),"Aprovado",IF(H3&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Turma!B4</f>
+        <v/>
+      </c>
+      <c r="C4" s="3">
+        <f>IFERROR(('Presença - Fev'!AK4+'Presença - Mar'!AK4+'Presença - Abr'!AK4+'Presença - Mai'!AK4+'Presença - Jun'!AK4+'Presença - Jul'!AK4+'Presença - Ago'!AK4+'Presença - Set'!AK4+'Presença - Out'!AK4+'Presença - Nov'!AK4)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'Notas - B1'!I4</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>'Notas - B2'!I4</f>
+        <v/>
+      </c>
+      <c r="F4" s="4">
+        <f>'Notas - B3'!I4</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>'Notas - B4'!I4</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>IFERROR(AVERAGE(D4:G4),"")</f>
+        <v/>
+      </c>
+      <c r="I4" s="2">
+        <f>IF(H4="","",IF(AND(H4&gt;=5,C4&gt;=0.75),"Aprovado",IF(H4&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Turma!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="3">
+        <f>IFERROR(('Presença - Fev'!AK5+'Presença - Mar'!AK5+'Presença - Abr'!AK5+'Presença - Mai'!AK5+'Presença - Jun'!AK5+'Presença - Jul'!AK5+'Presença - Ago'!AK5+'Presença - Set'!AK5+'Presença - Out'!AK5+'Presença - Nov'!AK5)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'Notas - B1'!I5</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>'Notas - B2'!I5</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>'Notas - B3'!I5</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>'Notas - B4'!I5</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>IFERROR(AVERAGE(D5:G5),"")</f>
+        <v/>
+      </c>
+      <c r="I5" s="2">
+        <f>IF(H5="","",IF(AND(H5&gt;=5,C5&gt;=0.75),"Aprovado",IF(H5&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Turma!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="3">
+        <f>IFERROR(('Presença - Fev'!AK6+'Presença - Mar'!AK6+'Presença - Abr'!AK6+'Presença - Mai'!AK6+'Presença - Jun'!AK6+'Presença - Jul'!AK6+'Presença - Ago'!AK6+'Presença - Set'!AK6+'Presença - Out'!AK6+'Presença - Nov'!AK6)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'Notas - B1'!I6</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'Notas - B2'!I6</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>'Notas - B3'!I6</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>'Notas - B4'!I6</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>IFERROR(AVERAGE(D6:G6),"")</f>
+        <v/>
+      </c>
+      <c r="I6" s="2">
+        <f>IF(H6="","",IF(AND(H6&gt;=5,C6&gt;=0.75),"Aprovado",IF(H6&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Turma!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="3">
+        <f>IFERROR(('Presença - Fev'!AK7+'Presença - Mar'!AK7+'Presença - Abr'!AK7+'Presença - Mai'!AK7+'Presença - Jun'!AK7+'Presença - Jul'!AK7+'Presença - Ago'!AK7+'Presença - Set'!AK7+'Presença - Out'!AK7+'Presença - Nov'!AK7)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>'Notas - B1'!I7</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>'Notas - B2'!I7</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>'Notas - B3'!I7</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>'Notas - B4'!I7</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>IFERROR(AVERAGE(D7:G7),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="2">
+        <f>IF(H7="","",IF(AND(H7&gt;=5,C7&gt;=0.75),"Aprovado",IF(H7&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Turma!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="3">
+        <f>IFERROR(('Presença - Fev'!AK8+'Presença - Mar'!AK8+'Presença - Abr'!AK8+'Presença - Mai'!AK8+'Presença - Jun'!AK8+'Presença - Jul'!AK8+'Presença - Ago'!AK8+'Presença - Set'!AK8+'Presença - Out'!AK8+'Presença - Nov'!AK8)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'Notas - B1'!I8</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>'Notas - B2'!I8</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>'Notas - B3'!I8</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>'Notas - B4'!I8</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>IFERROR(AVERAGE(D8:G8),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="2">
+        <f>IF(H8="","",IF(AND(H8&gt;=5,C8&gt;=0.75),"Aprovado",IF(H8&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Turma!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="3">
+        <f>IFERROR(('Presença - Fev'!AK9+'Presença - Mar'!AK9+'Presença - Abr'!AK9+'Presença - Mai'!AK9+'Presença - Jun'!AK9+'Presença - Jul'!AK9+'Presença - Ago'!AK9+'Presença - Set'!AK9+'Presença - Out'!AK9+'Presença - Nov'!AK9)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>'Notas - B1'!I9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>'Notas - B2'!I9</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>'Notas - B3'!I9</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>'Notas - B4'!I9</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>IFERROR(AVERAGE(D9:G9),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="2">
+        <f>IF(H9="","",IF(AND(H9&gt;=5,C9&gt;=0.75),"Aprovado",IF(H9&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Turma!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="3">
+        <f>IFERROR(('Presença - Fev'!AK10+'Presença - Mar'!AK10+'Presença - Abr'!AK10+'Presença - Mai'!AK10+'Presença - Jun'!AK10+'Presença - Jul'!AK10+'Presença - Ago'!AK10+'Presença - Set'!AK10+'Presença - Out'!AK10+'Presença - Nov'!AK10)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>'Notas - B1'!I10</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>'Notas - B2'!I10</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>'Notas - B3'!I10</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>'Notas - B4'!I10</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>IFERROR(AVERAGE(D10:G10),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="2">
+        <f>IF(H10="","",IF(AND(H10&gt;=5,C10&gt;=0.75),"Aprovado",IF(H10&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2">
+        <f>Turma!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="3">
+        <f>IFERROR(('Presença - Fev'!AK11+'Presença - Mar'!AK11+'Presença - Abr'!AK11+'Presença - Mai'!AK11+'Presença - Jun'!AK11+'Presença - Jul'!AK11+'Presença - Ago'!AK11+'Presença - Set'!AK11+'Presença - Out'!AK11+'Presença - Nov'!AK11)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>'Notas - B1'!I11</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>'Notas - B2'!I11</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>'Notas - B3'!I11</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>'Notas - B4'!I11</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>IFERROR(AVERAGE(D11:G11),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="2">
+        <f>IF(H11="","",IF(AND(H11&gt;=5,C11&gt;=0.75),"Aprovado",IF(H11&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2">
+        <f>Turma!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="3">
+        <f>IFERROR(('Presença - Fev'!AK12+'Presença - Mar'!AK12+'Presença - Abr'!AK12+'Presença - Mai'!AK12+'Presença - Jun'!AK12+'Presença - Jul'!AK12+'Presença - Ago'!AK12+'Presença - Set'!AK12+'Presença - Out'!AK12+'Presença - Nov'!AK12)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>'Notas - B1'!I12</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>'Notas - B2'!I12</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>'Notas - B3'!I12</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>'Notas - B4'!I12</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>IFERROR(AVERAGE(D12:G12),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="2">
+        <f>IF(H12="","",IF(AND(H12&gt;=5,C12&gt;=0.75),"Aprovado",IF(H12&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <f>Turma!B13</f>
+        <v/>
+      </c>
+      <c r="C13" s="3">
+        <f>IFERROR(('Presença - Fev'!AK13+'Presença - Mar'!AK13+'Presença - Abr'!AK13+'Presença - Mai'!AK13+'Presença - Jun'!AK13+'Presença - Jul'!AK13+'Presença - Ago'!AK13+'Presença - Set'!AK13+'Presença - Out'!AK13+'Presença - Nov'!AK13)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="4">
+        <f>'Notas - B1'!I13</f>
+        <v/>
+      </c>
+      <c r="E13" s="4">
+        <f>'Notas - B2'!I13</f>
+        <v/>
+      </c>
+      <c r="F13" s="4">
+        <f>'Notas - B3'!I13</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
+        <f>'Notas - B4'!I13</f>
+        <v/>
+      </c>
+      <c r="H13" s="4">
+        <f>IFERROR(AVERAGE(D13:G13),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="2">
+        <f>IF(H13="","",IF(AND(H13&gt;=5,C13&gt;=0.75),"Aprovado",IF(H13&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2">
+        <f>Turma!B14</f>
+        <v/>
+      </c>
+      <c r="C14" s="3">
+        <f>IFERROR(('Presença - Fev'!AK14+'Presença - Mar'!AK14+'Presença - Abr'!AK14+'Presença - Mai'!AK14+'Presença - Jun'!AK14+'Presença - Jul'!AK14+'Presença - Ago'!AK14+'Presença - Set'!AK14+'Presença - Out'!AK14+'Presença - Nov'!AK14)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="4">
+        <f>'Notas - B1'!I14</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>'Notas - B2'!I14</f>
+        <v/>
+      </c>
+      <c r="F14" s="4">
+        <f>'Notas - B3'!I14</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>'Notas - B4'!I14</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>IFERROR(AVERAGE(D14:G14),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="2">
+        <f>IF(H14="","",IF(AND(H14&gt;=5,C14&gt;=0.75),"Aprovado",IF(H14&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2">
+        <f>Turma!B15</f>
+        <v/>
+      </c>
+      <c r="C15" s="3">
+        <f>IFERROR(('Presença - Fev'!AK15+'Presença - Mar'!AK15+'Presença - Abr'!AK15+'Presença - Mai'!AK15+'Presença - Jun'!AK15+'Presença - Jul'!AK15+'Presença - Ago'!AK15+'Presença - Set'!AK15+'Presença - Out'!AK15+'Presença - Nov'!AK15)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="4">
+        <f>'Notas - B1'!I15</f>
+        <v/>
+      </c>
+      <c r="E15" s="4">
+        <f>'Notas - B2'!I15</f>
+        <v/>
+      </c>
+      <c r="F15" s="4">
+        <f>'Notas - B3'!I15</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>'Notas - B4'!I15</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>IFERROR(AVERAGE(D15:G15),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="2">
+        <f>IF(H15="","",IF(AND(H15&gt;=5,C15&gt;=0.75),"Aprovado",IF(H15&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2">
+        <f>Turma!B16</f>
+        <v/>
+      </c>
+      <c r="C16" s="3">
+        <f>IFERROR(('Presença - Fev'!AK16+'Presença - Mar'!AK16+'Presença - Abr'!AK16+'Presença - Mai'!AK16+'Presença - Jun'!AK16+'Presença - Jul'!AK16+'Presença - Ago'!AK16+'Presença - Set'!AK16+'Presença - Out'!AK16+'Presença - Nov'!AK16)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>'Notas - B1'!I16</f>
+        <v/>
+      </c>
+      <c r="E16" s="4">
+        <f>'Notas - B2'!I16</f>
+        <v/>
+      </c>
+      <c r="F16" s="4">
+        <f>'Notas - B3'!I16</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>'Notas - B4'!I16</f>
+        <v/>
+      </c>
+      <c r="H16" s="4">
+        <f>IFERROR(AVERAGE(D16:G16),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="2">
+        <f>IF(H16="","",IF(AND(H16&gt;=5,C16&gt;=0.75),"Aprovado",IF(H16&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2">
+        <f>Turma!B17</f>
+        <v/>
+      </c>
+      <c r="C17" s="3">
+        <f>IFERROR(('Presença - Fev'!AK17+'Presença - Mar'!AK17+'Presença - Abr'!AK17+'Presença - Mai'!AK17+'Presença - Jun'!AK17+'Presença - Jul'!AK17+'Presença - Ago'!AK17+'Presença - Set'!AK17+'Presença - Out'!AK17+'Presença - Nov'!AK17)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="4">
+        <f>'Notas - B1'!I17</f>
+        <v/>
+      </c>
+      <c r="E17" s="4">
+        <f>'Notas - B2'!I17</f>
+        <v/>
+      </c>
+      <c r="F17" s="4">
+        <f>'Notas - B3'!I17</f>
+        <v/>
+      </c>
+      <c r="G17" s="4">
+        <f>'Notas - B4'!I17</f>
+        <v/>
+      </c>
+      <c r="H17" s="4">
+        <f>IFERROR(AVERAGE(D17:G17),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="2">
+        <f>IF(H17="","",IF(AND(H17&gt;=5,C17&gt;=0.75),"Aprovado",IF(H17&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2">
+        <f>Turma!B18</f>
+        <v/>
+      </c>
+      <c r="C18" s="3">
+        <f>IFERROR(('Presença - Fev'!AK18+'Presença - Mar'!AK18+'Presença - Abr'!AK18+'Presença - Mai'!AK18+'Presença - Jun'!AK18+'Presença - Jul'!AK18+'Presença - Ago'!AK18+'Presença - Set'!AK18+'Presença - Out'!AK18+'Presença - Nov'!AK18)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="4">
+        <f>'Notas - B1'!I18</f>
+        <v/>
+      </c>
+      <c r="E18" s="4">
+        <f>'Notas - B2'!I18</f>
+        <v/>
+      </c>
+      <c r="F18" s="4">
+        <f>'Notas - B3'!I18</f>
+        <v/>
+      </c>
+      <c r="G18" s="4">
+        <f>'Notas - B4'!I18</f>
+        <v/>
+      </c>
+      <c r="H18" s="4">
+        <f>IFERROR(AVERAGE(D18:G18),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="2">
+        <f>IF(H18="","",IF(AND(H18&gt;=5,C18&gt;=0.75),"Aprovado",IF(H18&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2">
+        <f>Turma!B19</f>
+        <v/>
+      </c>
+      <c r="C19" s="3">
+        <f>IFERROR(('Presença - Fev'!AK19+'Presença - Mar'!AK19+'Presença - Abr'!AK19+'Presença - Mai'!AK19+'Presença - Jun'!AK19+'Presença - Jul'!AK19+'Presença - Ago'!AK19+'Presença - Set'!AK19+'Presença - Out'!AK19+'Presença - Nov'!AK19)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D19" s="4">
+        <f>'Notas - B1'!I19</f>
+        <v/>
+      </c>
+      <c r="E19" s="4">
+        <f>'Notas - B2'!I19</f>
+        <v/>
+      </c>
+      <c r="F19" s="4">
+        <f>'Notas - B3'!I19</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
+        <f>'Notas - B4'!I19</f>
+        <v/>
+      </c>
+      <c r="H19" s="4">
+        <f>IFERROR(AVERAGE(D19:G19),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="2">
+        <f>IF(H19="","",IF(AND(H19&gt;=5,C19&gt;=0.75),"Aprovado",IF(H19&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2">
+        <f>Turma!B20</f>
+        <v/>
+      </c>
+      <c r="C20" s="3">
+        <f>IFERROR(('Presença - Fev'!AK20+'Presença - Mar'!AK20+'Presença - Abr'!AK20+'Presença - Mai'!AK20+'Presença - Jun'!AK20+'Presença - Jul'!AK20+'Presença - Ago'!AK20+'Presença - Set'!AK20+'Presença - Out'!AK20+'Presença - Nov'!AK20)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="4">
+        <f>'Notas - B1'!I20</f>
+        <v/>
+      </c>
+      <c r="E20" s="4">
+        <f>'Notas - B2'!I20</f>
+        <v/>
+      </c>
+      <c r="F20" s="4">
+        <f>'Notas - B3'!I20</f>
+        <v/>
+      </c>
+      <c r="G20" s="4">
+        <f>'Notas - B4'!I20</f>
+        <v/>
+      </c>
+      <c r="H20" s="4">
+        <f>IFERROR(AVERAGE(D20:G20),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="2">
+        <f>IF(H20="","",IF(AND(H20&gt;=5,C20&gt;=0.75),"Aprovado",IF(H20&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2">
+        <f>Turma!B21</f>
+        <v/>
+      </c>
+      <c r="C21" s="3">
+        <f>IFERROR(('Presença - Fev'!AK21+'Presença - Mar'!AK21+'Presença - Abr'!AK21+'Presença - Mai'!AK21+'Presença - Jun'!AK21+'Presença - Jul'!AK21+'Presença - Ago'!AK21+'Presença - Set'!AK21+'Presença - Out'!AK21+'Presença - Nov'!AK21)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="4">
+        <f>'Notas - B1'!I21</f>
+        <v/>
+      </c>
+      <c r="E21" s="4">
+        <f>'Notas - B2'!I21</f>
+        <v/>
+      </c>
+      <c r="F21" s="4">
+        <f>'Notas - B3'!I21</f>
+        <v/>
+      </c>
+      <c r="G21" s="4">
+        <f>'Notas - B4'!I21</f>
+        <v/>
+      </c>
+      <c r="H21" s="4">
+        <f>IFERROR(AVERAGE(D21:G21),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="2">
+        <f>IF(H21="","",IF(AND(H21&gt;=5,C21&gt;=0.75),"Aprovado",IF(H21&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2">
+        <f>Turma!B22</f>
+        <v/>
+      </c>
+      <c r="C22" s="3">
+        <f>IFERROR(('Presença - Fev'!AK22+'Presença - Mar'!AK22+'Presença - Abr'!AK22+'Presença - Mai'!AK22+'Presença - Jun'!AK22+'Presença - Jul'!AK22+'Presença - Ago'!AK22+'Presença - Set'!AK22+'Presença - Out'!AK22+'Presença - Nov'!AK22)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>'Notas - B1'!I22</f>
+        <v/>
+      </c>
+      <c r="E22" s="4">
+        <f>'Notas - B2'!I22</f>
+        <v/>
+      </c>
+      <c r="F22" s="4">
+        <f>'Notas - B3'!I22</f>
+        <v/>
+      </c>
+      <c r="G22" s="4">
+        <f>'Notas - B4'!I22</f>
+        <v/>
+      </c>
+      <c r="H22" s="4">
+        <f>IFERROR(AVERAGE(D22:G22),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="2">
+        <f>IF(H22="","",IF(AND(H22&gt;=5,C22&gt;=0.75),"Aprovado",IF(H22&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2">
+        <f>Turma!B23</f>
+        <v/>
+      </c>
+      <c r="C23" s="3">
+        <f>IFERROR(('Presença - Fev'!AK23+'Presença - Mar'!AK23+'Presença - Abr'!AK23+'Presença - Mai'!AK23+'Presença - Jun'!AK23+'Presença - Jul'!AK23+'Presença - Ago'!AK23+'Presença - Set'!AK23+'Presença - Out'!AK23+'Presença - Nov'!AK23)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D23" s="4">
+        <f>'Notas - B1'!I23</f>
+        <v/>
+      </c>
+      <c r="E23" s="4">
+        <f>'Notas - B2'!I23</f>
+        <v/>
+      </c>
+      <c r="F23" s="4">
+        <f>'Notas - B3'!I23</f>
+        <v/>
+      </c>
+      <c r="G23" s="4">
+        <f>'Notas - B4'!I23</f>
+        <v/>
+      </c>
+      <c r="H23" s="4">
+        <f>IFERROR(AVERAGE(D23:G23),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="2">
+        <f>IF(H23="","",IF(AND(H23&gt;=5,C23&gt;=0.75),"Aprovado",IF(H23&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2">
+        <f>Turma!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="3">
+        <f>IFERROR(('Presença - Fev'!AK24+'Presença - Mar'!AK24+'Presença - Abr'!AK24+'Presença - Mai'!AK24+'Presença - Jun'!AK24+'Presença - Jul'!AK24+'Presença - Ago'!AK24+'Presença - Set'!AK24+'Presença - Out'!AK24+'Presença - Nov'!AK24)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="4">
+        <f>'Notas - B1'!I24</f>
+        <v/>
+      </c>
+      <c r="E24" s="4">
+        <f>'Notas - B2'!I24</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>'Notas - B3'!I24</f>
+        <v/>
+      </c>
+      <c r="G24" s="4">
+        <f>'Notas - B4'!I24</f>
+        <v/>
+      </c>
+      <c r="H24" s="4">
+        <f>IFERROR(AVERAGE(D24:G24),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="2">
+        <f>IF(H24="","",IF(AND(H24&gt;=5,C24&gt;=0.75),"Aprovado",IF(H24&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2">
+        <f>Turma!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="3">
+        <f>IFERROR(('Presença - Fev'!AK25+'Presença - Mar'!AK25+'Presença - Abr'!AK25+'Presença - Mai'!AK25+'Presença - Jun'!AK25+'Presença - Jul'!AK25+'Presença - Ago'!AK25+'Presença - Set'!AK25+'Presença - Out'!AK25+'Presença - Nov'!AK25)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="4">
+        <f>'Notas - B1'!I25</f>
+        <v/>
+      </c>
+      <c r="E25" s="4">
+        <f>'Notas - B2'!I25</f>
+        <v/>
+      </c>
+      <c r="F25" s="4">
+        <f>'Notas - B3'!I25</f>
+        <v/>
+      </c>
+      <c r="G25" s="4">
+        <f>'Notas - B4'!I25</f>
+        <v/>
+      </c>
+      <c r="H25" s="4">
+        <f>IFERROR(AVERAGE(D25:G25),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="2">
+        <f>IF(H25="","",IF(AND(H25&gt;=5,C25&gt;=0.75),"Aprovado",IF(H25&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2">
+        <f>Turma!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="3">
+        <f>IFERROR(('Presença - Fev'!AK26+'Presença - Mar'!AK26+'Presença - Abr'!AK26+'Presença - Mai'!AK26+'Presença - Jun'!AK26+'Presença - Jul'!AK26+'Presença - Ago'!AK26+'Presença - Set'!AK26+'Presença - Out'!AK26+'Presença - Nov'!AK26)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="4">
+        <f>'Notas - B1'!I26</f>
+        <v/>
+      </c>
+      <c r="E26" s="4">
+        <f>'Notas - B2'!I26</f>
+        <v/>
+      </c>
+      <c r="F26" s="4">
+        <f>'Notas - B3'!I26</f>
+        <v/>
+      </c>
+      <c r="G26" s="4">
+        <f>'Notas - B4'!I26</f>
+        <v/>
+      </c>
+      <c r="H26" s="4">
+        <f>IFERROR(AVERAGE(D26:G26),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="2">
+        <f>IF(H26="","",IF(AND(H26&gt;=5,C26&gt;=0.75),"Aprovado",IF(H26&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2">
+        <f>Turma!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="3">
+        <f>IFERROR(('Presença - Fev'!AK27+'Presença - Mar'!AK27+'Presença - Abr'!AK27+'Presença - Mai'!AK27+'Presença - Jun'!AK27+'Presença - Jul'!AK27+'Presença - Ago'!AK27+'Presença - Set'!AK27+'Presença - Out'!AK27+'Presença - Nov'!AK27)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>'Notas - B1'!I27</f>
+        <v/>
+      </c>
+      <c r="E27" s="4">
+        <f>'Notas - B2'!I27</f>
+        <v/>
+      </c>
+      <c r="F27" s="4">
+        <f>'Notas - B3'!I27</f>
+        <v/>
+      </c>
+      <c r="G27" s="4">
+        <f>'Notas - B4'!I27</f>
+        <v/>
+      </c>
+      <c r="H27" s="4">
+        <f>IFERROR(AVERAGE(D27:G27),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="2">
+        <f>IF(H27="","",IF(AND(H27&gt;=5,C27&gt;=0.75),"Aprovado",IF(H27&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2">
+        <f>Turma!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="3">
+        <f>IFERROR(('Presença - Fev'!AK28+'Presença - Mar'!AK28+'Presença - Abr'!AK28+'Presença - Mai'!AK28+'Presença - Jun'!AK28+'Presença - Jul'!AK28+'Presença - Ago'!AK28+'Presença - Set'!AK28+'Presença - Out'!AK28+'Presença - Nov'!AK28)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="4">
+        <f>'Notas - B1'!I28</f>
+        <v/>
+      </c>
+      <c r="E28" s="4">
+        <f>'Notas - B2'!I28</f>
+        <v/>
+      </c>
+      <c r="F28" s="4">
+        <f>'Notas - B3'!I28</f>
+        <v/>
+      </c>
+      <c r="G28" s="4">
+        <f>'Notas - B4'!I28</f>
+        <v/>
+      </c>
+      <c r="H28" s="4">
+        <f>IFERROR(AVERAGE(D28:G28),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="2">
+        <f>IF(H28="","",IF(AND(H28&gt;=5,C28&gt;=0.75),"Aprovado",IF(H28&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2">
+        <f>Turma!B29</f>
+        <v/>
+      </c>
+      <c r="C29" s="3">
+        <f>IFERROR(('Presença - Fev'!AK29+'Presença - Mar'!AK29+'Presença - Abr'!AK29+'Presença - Mai'!AK29+'Presença - Jun'!AK29+'Presença - Jul'!AK29+'Presença - Ago'!AK29+'Presença - Set'!AK29+'Presença - Out'!AK29+'Presença - Nov'!AK29)/10,"")</f>
+        <v/>
+      </c>
+      <c r="D29" s="4">
+        <f>'Notas - B1'!I29</f>
+        <v/>
+      </c>
+      <c r="E29" s="4">
+        <f>'Notas - B2'!I29</f>
+        <v/>
+      </c>
+      <c r="F29" s="4">
+        <f>'Notas - B3'!I29</f>
+        <v/>
+      </c>
+      <c r="G29" s="4">
+        <f>'Notas - B4'!I29</f>
+        <v/>
+      </c>
+      <c r="H29" s="4">
+        <f>IFERROR(AVERAGE(D29:G29),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="2">
+        <f>IF(H29="","",IF(AND(H29&gt;=5,C29&gt;=0.75),"Aprovado",IF(H29&gt;=5,"Rec. Freq.","Recuperação")))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I3:I29">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Aprovado"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+      <formula>"Recuperação"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Rec. Freq."</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix: corrigir off-by-one Resumo Anual e melhorias de qualidade
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diario-de-classe.xlsx
+++ b/diario-de-classe.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -107,7 +107,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -5069,7 +5068,7 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>5</formula>
-      <formula>6.9</formula>
+      <formula>6.99</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
       <formula>7</formula>
@@ -5667,7 +5666,7 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>5</formula>
-      <formula>6.9</formula>
+      <formula>6.99</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
       <formula>7</formula>
@@ -6265,7 +6264,7 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>5</formula>
-      <formula>6.9</formula>
+      <formula>6.99</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
       <formula>7</formula>
@@ -6863,7 +6862,7 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>5</formula>
-      <formula>6.9</formula>
+      <formula>6.99</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
       <formula>7</formula>
@@ -7478,905 +7477,905 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="5" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="5" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="5" t="n"/>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="5" t="n"/>
-      <c r="G46" s="5" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="5" t="n"/>
-      <c r="G52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="5" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="5" t="n"/>
-      <c r="G54" s="5" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="5" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="5" t="n"/>
-      <c r="G55" s="5" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="5" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="n"/>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="5" t="n"/>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="5" t="n"/>
-      <c r="G57" s="5" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="5" t="n"/>
-      <c r="D58" s="5" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="5" t="n"/>
-      <c r="G58" s="5" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="5" t="n"/>
-      <c r="D59" s="5" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="5" t="n"/>
-      <c r="D60" s="5" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="5" t="n"/>
-      <c r="G60" s="5" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="5" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="5" t="n"/>
-      <c r="G61" s="5" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="5" t="n"/>
-      <c r="D62" s="5" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="5" t="n"/>
-      <c r="G62" s="5" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="5" t="n"/>
-      <c r="D63" s="5" t="n"/>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="5" t="n"/>
-      <c r="G63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="5" t="n"/>
-      <c r="D64" s="5" t="n"/>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="5" t="n"/>
-      <c r="G64" s="5" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="5" t="n"/>
-      <c r="D65" s="5" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="5" t="n"/>
-      <c r="G65" s="5" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="n"/>
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="5" t="n"/>
-      <c r="D66" s="5" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="5" t="n"/>
-      <c r="G66" s="5" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="n"/>
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="5" t="n"/>
-      <c r="D67" s="5" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="5" t="n"/>
-      <c r="G67" s="5" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="n"/>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="5" t="n"/>
-      <c r="D68" s="5" t="n"/>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="5" t="n"/>
-      <c r="G68" s="5" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="5" t="n"/>
-      <c r="D69" s="5" t="n"/>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="5" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="n"/>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="5" t="n"/>
-      <c r="D70" s="5" t="n"/>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="5" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="n"/>
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="5" t="n"/>
-      <c r="D71" s="5" t="n"/>
-      <c r="E71" s="2" t="n"/>
-      <c r="F71" s="5" t="n"/>
-      <c r="G71" s="5" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="n"/>
-      <c r="B72" s="2" t="n"/>
-      <c r="C72" s="5" t="n"/>
-      <c r="D72" s="5" t="n"/>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="5" t="n"/>
-      <c r="G72" s="5" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="n"/>
-      <c r="B73" s="2" t="n"/>
-      <c r="C73" s="5" t="n"/>
-      <c r="D73" s="5" t="n"/>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="5" t="n"/>
-      <c r="G73" s="5" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="n"/>
-      <c r="B74" s="2" t="n"/>
-      <c r="C74" s="5" t="n"/>
-      <c r="D74" s="5" t="n"/>
-      <c r="E74" s="2" t="n"/>
-      <c r="F74" s="5" t="n"/>
-      <c r="G74" s="5" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="n"/>
-      <c r="B75" s="2" t="n"/>
-      <c r="C75" s="5" t="n"/>
-      <c r="D75" s="5" t="n"/>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="5" t="n"/>
-      <c r="G75" s="5" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="n"/>
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="5" t="n"/>
-      <c r="D76" s="5" t="n"/>
-      <c r="E76" s="2" t="n"/>
-      <c r="F76" s="5" t="n"/>
-      <c r="G76" s="5" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="n"/>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="5" t="n"/>
-      <c r="D77" s="5" t="n"/>
-      <c r="E77" s="2" t="n"/>
-      <c r="F77" s="5" t="n"/>
-      <c r="G77" s="5" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="n"/>
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="5" t="n"/>
-      <c r="D78" s="5" t="n"/>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="5" t="n"/>
-      <c r="G78" s="5" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="n"/>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="5" t="n"/>
-      <c r="D79" s="5" t="n"/>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="5" t="n"/>
-      <c r="G79" s="5" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n"/>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="5" t="n"/>
-      <c r="D80" s="5" t="n"/>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="5" t="n"/>
-      <c r="G80" s="5" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="n"/>
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="5" t="n"/>
-      <c r="D81" s="5" t="n"/>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="5" t="n"/>
-      <c r="G81" s="5" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="n"/>
-      <c r="B82" s="2" t="n"/>
-      <c r="C82" s="5" t="n"/>
-      <c r="D82" s="5" t="n"/>
-      <c r="E82" s="2" t="n"/>
-      <c r="F82" s="5" t="n"/>
-      <c r="G82" s="5" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="n"/>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="5" t="n"/>
-      <c r="D83" s="5" t="n"/>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="5" t="n"/>
-      <c r="G83" s="5" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n"/>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="5" t="n"/>
-      <c r="D84" s="5" t="n"/>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="5" t="n"/>
-      <c r="G84" s="5" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="n"/>
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="5" t="n"/>
-      <c r="D85" s="5" t="n"/>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="5" t="n"/>
-      <c r="G85" s="5" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="n"/>
-      <c r="B86" s="2" t="n"/>
-      <c r="C86" s="5" t="n"/>
-      <c r="D86" s="5" t="n"/>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="5" t="n"/>
-      <c r="G86" s="5" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="5" t="n"/>
-      <c r="D87" s="5" t="n"/>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="5" t="n"/>
-      <c r="G87" s="5" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="n"/>
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="5" t="n"/>
-      <c r="D88" s="5" t="n"/>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="5" t="n"/>
-      <c r="G88" s="5" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="n"/>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="5" t="n"/>
-      <c r="D89" s="5" t="n"/>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="5" t="n"/>
-      <c r="G89" s="5" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="n"/>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="5" t="n"/>
-      <c r="D90" s="5" t="n"/>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="5" t="n"/>
-      <c r="G90" s="5" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="5" t="n"/>
-      <c r="D91" s="5" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="5" t="n"/>
-      <c r="G91" s="5" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="n"/>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="5" t="n"/>
-      <c r="D92" s="5" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="5" t="n"/>
-      <c r="G92" s="5" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="n"/>
-      <c r="B93" s="2" t="n"/>
-      <c r="C93" s="5" t="n"/>
-      <c r="D93" s="5" t="n"/>
-      <c r="E93" s="2" t="n"/>
-      <c r="F93" s="5" t="n"/>
-      <c r="G93" s="5" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="n"/>
-      <c r="B94" s="2" t="n"/>
-      <c r="C94" s="5" t="n"/>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="5" t="n"/>
-      <c r="G94" s="5" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="n"/>
-      <c r="B95" s="2" t="n"/>
-      <c r="C95" s="5" t="n"/>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="2" t="n"/>
-      <c r="F95" s="5" t="n"/>
-      <c r="G95" s="5" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="n"/>
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="5" t="n"/>
-      <c r="D96" s="5" t="n"/>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="5" t="n"/>
-      <c r="G96" s="5" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="n"/>
-      <c r="B97" s="2" t="n"/>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="2" t="n"/>
-      <c r="F97" s="5" t="n"/>
-      <c r="G97" s="5" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="n"/>
-      <c r="B98" s="2" t="n"/>
-      <c r="C98" s="5" t="n"/>
-      <c r="D98" s="5" t="n"/>
-      <c r="E98" s="2" t="n"/>
-      <c r="F98" s="5" t="n"/>
-      <c r="G98" s="5" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="n"/>
-      <c r="B99" s="2" t="n"/>
-      <c r="C99" s="5" t="n"/>
-      <c r="D99" s="5" t="n"/>
-      <c r="E99" s="2" t="n"/>
-      <c r="F99" s="5" t="n"/>
-      <c r="G99" s="5" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="n"/>
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="5" t="n"/>
-      <c r="D100" s="5" t="n"/>
-      <c r="E100" s="2" t="n"/>
-      <c r="F100" s="5" t="n"/>
-      <c r="G100" s="5" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="n"/>
-      <c r="B101" s="2" t="n"/>
-      <c r="C101" s="5" t="n"/>
-      <c r="D101" s="5" t="n"/>
-      <c r="E101" s="2" t="n"/>
-      <c r="F101" s="5" t="n"/>
-      <c r="G101" s="5" t="n"/>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="6" t="n"/>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="5" t="n"/>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="5" t="n"/>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="6" t="n"/>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="6" t="n"/>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="5" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="6" t="n"/>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="6" t="n"/>
+    </row>
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="6" t="n"/>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="5" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="5" t="n"/>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="6" t="n"/>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="6" t="n"/>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="5" t="n"/>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="6" t="n"/>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="5" t="n"/>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="6" t="n"/>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="5" t="n"/>
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="5" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="6" t="n"/>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="5" t="n"/>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="5" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="6" t="n"/>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="5" t="n"/>
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="5" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="6" t="n"/>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="6" t="n"/>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="5" t="n"/>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="6" t="n"/>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="5" t="n"/>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="6" t="n"/>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="5" t="n"/>
+      <c r="B64" s="5" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="5" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="6" t="n"/>
+    </row>
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="5" t="n"/>
+      <c r="B65" s="5" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="5" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="6" t="n"/>
+    </row>
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="5" t="n"/>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="6" t="n"/>
+    </row>
+    <row r="67" ht="40" customHeight="1">
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="5" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="5" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n"/>
+    </row>
+    <row r="68" ht="40" customHeight="1">
+      <c r="A68" s="5" t="n"/>
+      <c r="B68" s="5" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="5" t="n"/>
+      <c r="F68" s="6" t="n"/>
+      <c r="G68" s="6" t="n"/>
+    </row>
+    <row r="69" ht="40" customHeight="1">
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="5" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="5" t="n"/>
+      <c r="F69" s="6" t="n"/>
+      <c r="G69" s="6" t="n"/>
+    </row>
+    <row r="70" ht="40" customHeight="1">
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="5" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="5" t="n"/>
+      <c r="F70" s="6" t="n"/>
+      <c r="G70" s="6" t="n"/>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="5" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="5" t="n"/>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="6" t="n"/>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="5" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="5" t="n"/>
+      <c r="F72" s="6" t="n"/>
+      <c r="G72" s="6" t="n"/>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="6" t="n"/>
+      <c r="E73" s="5" t="n"/>
+      <c r="F73" s="6" t="n"/>
+      <c r="G73" s="6" t="n"/>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="5" t="n"/>
+      <c r="F74" s="6" t="n"/>
+      <c r="G74" s="6" t="n"/>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="5" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="5" t="n"/>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="6" t="n"/>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="5" t="n"/>
+      <c r="B76" s="5" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="5" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="5" t="n"/>
+      <c r="B77" s="5" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="5" t="n"/>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="5" t="n"/>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="6" t="n"/>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="5" t="n"/>
+      <c r="B79" s="5" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="5" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="5" t="n"/>
+      <c r="B80" s="5" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="5" t="n"/>
+      <c r="F80" s="6" t="n"/>
+      <c r="G80" s="6" t="n"/>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="5" t="n"/>
+      <c r="B81" s="5" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="5" t="n"/>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="6" t="n"/>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="5" t="n"/>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="5" t="n"/>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="6" t="n"/>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="5" t="n"/>
+      <c r="B83" s="5" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="5" t="n"/>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="6" t="n"/>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="5" t="n"/>
+      <c r="B84" s="5" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="5" t="n"/>
+      <c r="F84" s="6" t="n"/>
+      <c r="G84" s="6" t="n"/>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="5" t="n"/>
+      <c r="B85" s="5" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="5" t="n"/>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="6" t="n"/>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="5" t="n"/>
+      <c r="B86" s="5" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="5" t="n"/>
+      <c r="F86" s="6" t="n"/>
+      <c r="G86" s="6" t="n"/>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="5" t="n"/>
+      <c r="B87" s="5" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="5" t="n"/>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n"/>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="5" t="n"/>
+      <c r="B88" s="5" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="5" t="n"/>
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="6" t="n"/>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="5" t="n"/>
+      <c r="B89" s="5" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="5" t="n"/>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="6" t="n"/>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="5" t="n"/>
+      <c r="B90" s="5" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="5" t="n"/>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="6" t="n"/>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="5" t="n"/>
+      <c r="B91" s="5" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="5" t="n"/>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="6" t="n"/>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="5" t="n"/>
+      <c r="B92" s="5" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="5" t="n"/>
+      <c r="F92" s="6" t="n"/>
+      <c r="G92" s="6" t="n"/>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="5" t="n"/>
+      <c r="B93" s="5" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="5" t="n"/>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="6" t="n"/>
+    </row>
+    <row r="94" ht="40" customHeight="1">
+      <c r="A94" s="5" t="n"/>
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="5" t="n"/>
+      <c r="F94" s="6" t="n"/>
+      <c r="G94" s="6" t="n"/>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="A95" s="5" t="n"/>
+      <c r="B95" s="5" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="5" t="n"/>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="6" t="n"/>
+    </row>
+    <row r="96" ht="40" customHeight="1">
+      <c r="A96" s="5" t="n"/>
+      <c r="B96" s="5" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="5" t="n"/>
+      <c r="F96" s="6" t="n"/>
+      <c r="G96" s="6" t="n"/>
+    </row>
+    <row r="97" ht="40" customHeight="1">
+      <c r="A97" s="5" t="n"/>
+      <c r="B97" s="5" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="5" t="n"/>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+    </row>
+    <row r="98" ht="40" customHeight="1">
+      <c r="A98" s="5" t="n"/>
+      <c r="B98" s="5" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="5" t="n"/>
+      <c r="F98" s="6" t="n"/>
+      <c r="G98" s="6" t="n"/>
+    </row>
+    <row r="99" ht="40" customHeight="1">
+      <c r="A99" s="5" t="n"/>
+      <c r="B99" s="5" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="5" t="n"/>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+    </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="5" t="n"/>
+      <c r="B100" s="5" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="5" t="n"/>
+      <c r="F100" s="6" t="n"/>
+      <c r="G100" s="6" t="n"/>
+    </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="5" t="n"/>
+      <c r="B101" s="5" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="5" t="n"/>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8428,704 +8427,704 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="6" t="n"/>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="7" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
     </row>
     <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
     </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
     </row>
     <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
     </row>
     <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
     </row>
     <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
     </row>
     <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
     </row>
     <row r="29" ht="40" customHeight="1">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
     </row>
     <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
     </row>
     <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
     </row>
     <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
     </row>
     <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
+      <c r="A33" s="5" t="n"/>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
     </row>
     <row r="34" ht="40" customHeight="1">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
+      <c r="A34" s="5" t="n"/>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
     </row>
     <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
     </row>
     <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
     </row>
     <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
     </row>
     <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
     </row>
     <row r="39" ht="40" customHeight="1">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
     </row>
     <row r="40" ht="40" customHeight="1">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
     </row>
     <row r="41" ht="40" customHeight="1">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="7" t="n"/>
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
     </row>
     <row r="42" ht="40" customHeight="1">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
-      <c r="E42" s="7" t="n"/>
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
     </row>
     <row r="43" ht="40" customHeight="1">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="7" t="n"/>
-      <c r="D43" s="7" t="n"/>
-      <c r="E43" s="7" t="n"/>
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
     </row>
     <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="7" t="n"/>
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="5" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
     </row>
     <row r="45" ht="40" customHeight="1">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="7" t="n"/>
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
     </row>
     <row r="46" ht="40" customHeight="1">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="7" t="n"/>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="7" t="n"/>
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
     </row>
     <row r="47" ht="40" customHeight="1">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
-      <c r="E47" s="7" t="n"/>
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
     </row>
     <row r="48" ht="40" customHeight="1">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
     </row>
     <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
     </row>
     <row r="50" ht="40" customHeight="1">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="n"/>
-      <c r="E50" s="7" t="n"/>
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
     </row>
     <row r="51" ht="40" customHeight="1">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="7" t="n"/>
-      <c r="D51" s="7" t="n"/>
-      <c r="E51" s="7" t="n"/>
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
     </row>
     <row r="52" ht="40" customHeight="1">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="n"/>
-      <c r="E52" s="7" t="n"/>
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
     </row>
     <row r="53" ht="40" customHeight="1">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="7" t="n"/>
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
     </row>
     <row r="54" ht="40" customHeight="1">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="7" t="n"/>
+      <c r="A54" s="5" t="n"/>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
     </row>
     <row r="55" ht="40" customHeight="1">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="n"/>
-      <c r="E55" s="7" t="n"/>
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
     </row>
     <row r="56" ht="40" customHeight="1">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="7" t="n"/>
-      <c r="D56" s="7" t="n"/>
-      <c r="E56" s="7" t="n"/>
+      <c r="A56" s="5" t="n"/>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
     </row>
     <row r="57" ht="40" customHeight="1">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="7" t="n"/>
-      <c r="D57" s="7" t="n"/>
-      <c r="E57" s="7" t="n"/>
+      <c r="A57" s="5" t="n"/>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
     </row>
     <row r="58" ht="40" customHeight="1">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="7" t="n"/>
-      <c r="D58" s="7" t="n"/>
-      <c r="E58" s="7" t="n"/>
+      <c r="A58" s="5" t="n"/>
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
     </row>
     <row r="59" ht="40" customHeight="1">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
-      <c r="E59" s="7" t="n"/>
+      <c r="A59" s="5" t="n"/>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
     </row>
     <row r="60" ht="40" customHeight="1">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="n"/>
-      <c r="E60" s="7" t="n"/>
+      <c r="A60" s="5" t="n"/>
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
     </row>
     <row r="61" ht="40" customHeight="1">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="n"/>
-      <c r="E61" s="7" t="n"/>
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
     </row>
     <row r="62" ht="40" customHeight="1">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="7" t="n"/>
-      <c r="D62" s="7" t="n"/>
-      <c r="E62" s="7" t="n"/>
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
     </row>
     <row r="63" ht="40" customHeight="1">
-      <c r="A63" s="6" t="n"/>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
-      <c r="E63" s="7" t="n"/>
+      <c r="A63" s="5" t="n"/>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
     </row>
     <row r="64" ht="40" customHeight="1">
-      <c r="A64" s="6" t="n"/>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="n"/>
-      <c r="E64" s="7" t="n"/>
+      <c r="A64" s="5" t="n"/>
+      <c r="B64" s="5" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
     </row>
     <row r="65" ht="40" customHeight="1">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
-      <c r="E65" s="7" t="n"/>
+      <c r="A65" s="5" t="n"/>
+      <c r="B65" s="5" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
     </row>
     <row r="66" ht="40" customHeight="1">
-      <c r="A66" s="6" t="n"/>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="7" t="n"/>
-      <c r="D66" s="7" t="n"/>
-      <c r="E66" s="7" t="n"/>
+      <c r="A66" s="5" t="n"/>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
     </row>
     <row r="67" ht="40" customHeight="1">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
-      <c r="E67" s="7" t="n"/>
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="5" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
     </row>
     <row r="68" ht="40" customHeight="1">
-      <c r="A68" s="6" t="n"/>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
-      <c r="E68" s="7" t="n"/>
+      <c r="A68" s="5" t="n"/>
+      <c r="B68" s="5" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
     </row>
     <row r="69" ht="40" customHeight="1">
-      <c r="A69" s="6" t="n"/>
-      <c r="B69" s="6" t="n"/>
-      <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="n"/>
-      <c r="E69" s="7" t="n"/>
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="5" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="6" t="n"/>
     </row>
     <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="6" t="n"/>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="5" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
     </row>
     <row r="71" ht="40" customHeight="1">
-      <c r="A71" s="6" t="n"/>
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
-      <c r="E71" s="7" t="n"/>
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="5" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
     </row>
     <row r="72" ht="40" customHeight="1">
-      <c r="A72" s="6" t="n"/>
-      <c r="B72" s="6" t="n"/>
-      <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="n"/>
-      <c r="E72" s="7" t="n"/>
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="5" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="6" t="n"/>
     </row>
     <row r="73" ht="40" customHeight="1">
-      <c r="A73" s="6" t="n"/>
-      <c r="B73" s="6" t="n"/>
-      <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
-      <c r="E73" s="7" t="n"/>
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="6" t="n"/>
+      <c r="E73" s="6" t="n"/>
     </row>
     <row r="74" ht="40" customHeight="1">
-      <c r="A74" s="6" t="n"/>
-      <c r="B74" s="6" t="n"/>
-      <c r="C74" s="7" t="n"/>
-      <c r="D74" s="7" t="n"/>
-      <c r="E74" s="7" t="n"/>
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="6" t="n"/>
     </row>
     <row r="75" ht="40" customHeight="1">
-      <c r="A75" s="6" t="n"/>
-      <c r="B75" s="6" t="n"/>
-      <c r="C75" s="7" t="n"/>
-      <c r="D75" s="7" t="n"/>
-      <c r="E75" s="7" t="n"/>
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="5" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
     </row>
     <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="6" t="n"/>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="n"/>
-      <c r="E76" s="7" t="n"/>
+      <c r="A76" s="5" t="n"/>
+      <c r="B76" s="5" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
     </row>
     <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="6" t="n"/>
-      <c r="B77" s="6" t="n"/>
-      <c r="C77" s="7" t="n"/>
-      <c r="D77" s="7" t="n"/>
-      <c r="E77" s="7" t="n"/>
+      <c r="A77" s="5" t="n"/>
+      <c r="B77" s="5" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
     </row>
     <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="6" t="n"/>
-      <c r="B78" s="6" t="n"/>
-      <c r="C78" s="7" t="n"/>
-      <c r="D78" s="7" t="n"/>
-      <c r="E78" s="7" t="n"/>
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
     </row>
     <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="6" t="n"/>
-      <c r="B79" s="6" t="n"/>
-      <c r="C79" s="7" t="n"/>
-      <c r="D79" s="7" t="n"/>
-      <c r="E79" s="7" t="n"/>
+      <c r="A79" s="5" t="n"/>
+      <c r="B79" s="5" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
     </row>
     <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="6" t="n"/>
-      <c r="B80" s="6" t="n"/>
-      <c r="C80" s="7" t="n"/>
-      <c r="D80" s="7" t="n"/>
-      <c r="E80" s="7" t="n"/>
+      <c r="A80" s="5" t="n"/>
+      <c r="B80" s="5" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="6" t="n"/>
     </row>
     <row r="81" ht="40" customHeight="1">
-      <c r="A81" s="6" t="n"/>
-      <c r="B81" s="6" t="n"/>
-      <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="n"/>
-      <c r="E81" s="7" t="n"/>
+      <c r="A81" s="5" t="n"/>
+      <c r="B81" s="5" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="6" t="n"/>
     </row>
     <row r="82" ht="40" customHeight="1">
-      <c r="A82" s="6" t="n"/>
-      <c r="B82" s="6" t="n"/>
-      <c r="C82" s="7" t="n"/>
-      <c r="D82" s="7" t="n"/>
-      <c r="E82" s="7" t="n"/>
+      <c r="A82" s="5" t="n"/>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
     </row>
     <row r="83" ht="40" customHeight="1">
-      <c r="A83" s="6" t="n"/>
-      <c r="B83" s="6" t="n"/>
-      <c r="C83" s="7" t="n"/>
-      <c r="D83" s="7" t="n"/>
-      <c r="E83" s="7" t="n"/>
+      <c r="A83" s="5" t="n"/>
+      <c r="B83" s="5" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
     </row>
     <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="6" t="n"/>
-      <c r="B84" s="6" t="n"/>
-      <c r="C84" s="7" t="n"/>
-      <c r="D84" s="7" t="n"/>
-      <c r="E84" s="7" t="n"/>
+      <c r="A84" s="5" t="n"/>
+      <c r="B84" s="5" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="6" t="n"/>
     </row>
     <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="6" t="n"/>
-      <c r="B85" s="6" t="n"/>
-      <c r="C85" s="7" t="n"/>
-      <c r="D85" s="7" t="n"/>
-      <c r="E85" s="7" t="n"/>
+      <c r="A85" s="5" t="n"/>
+      <c r="B85" s="5" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
     </row>
     <row r="86" ht="40" customHeight="1">
-      <c r="A86" s="6" t="n"/>
-      <c r="B86" s="6" t="n"/>
-      <c r="C86" s="7" t="n"/>
-      <c r="D86" s="7" t="n"/>
-      <c r="E86" s="7" t="n"/>
+      <c r="A86" s="5" t="n"/>
+      <c r="B86" s="5" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="6" t="n"/>
     </row>
     <row r="87" ht="40" customHeight="1">
-      <c r="A87" s="6" t="n"/>
-      <c r="B87" s="6" t="n"/>
-      <c r="C87" s="7" t="n"/>
-      <c r="D87" s="7" t="n"/>
-      <c r="E87" s="7" t="n"/>
+      <c r="A87" s="5" t="n"/>
+      <c r="B87" s="5" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="6" t="n"/>
     </row>
     <row r="88" ht="40" customHeight="1">
-      <c r="A88" s="6" t="n"/>
-      <c r="B88" s="6" t="n"/>
-      <c r="C88" s="7" t="n"/>
-      <c r="D88" s="7" t="n"/>
-      <c r="E88" s="7" t="n"/>
+      <c r="A88" s="5" t="n"/>
+      <c r="B88" s="5" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="6" t="n"/>
     </row>
     <row r="89" ht="40" customHeight="1">
-      <c r="A89" s="6" t="n"/>
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="7" t="n"/>
-      <c r="D89" s="7" t="n"/>
-      <c r="E89" s="7" t="n"/>
+      <c r="A89" s="5" t="n"/>
+      <c r="B89" s="5" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
     </row>
     <row r="90" ht="40" customHeight="1">
-      <c r="A90" s="6" t="n"/>
-      <c r="B90" s="6" t="n"/>
-      <c r="C90" s="7" t="n"/>
-      <c r="D90" s="7" t="n"/>
-      <c r="E90" s="7" t="n"/>
+      <c r="A90" s="5" t="n"/>
+      <c r="B90" s="5" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
     </row>
     <row r="91" ht="40" customHeight="1">
-      <c r="A91" s="6" t="n"/>
-      <c r="B91" s="6" t="n"/>
-      <c r="C91" s="7" t="n"/>
-      <c r="D91" s="7" t="n"/>
-      <c r="E91" s="7" t="n"/>
+      <c r="A91" s="5" t="n"/>
+      <c r="B91" s="5" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="6" t="n"/>
     </row>
     <row r="92" ht="40" customHeight="1">
-      <c r="A92" s="6" t="n"/>
-      <c r="B92" s="6" t="n"/>
-      <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
-      <c r="E92" s="7" t="n"/>
+      <c r="A92" s="5" t="n"/>
+      <c r="B92" s="5" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="6" t="n"/>
     </row>
     <row r="93" ht="40" customHeight="1">
-      <c r="A93" s="6" t="n"/>
-      <c r="B93" s="6" t="n"/>
-      <c r="C93" s="7" t="n"/>
-      <c r="D93" s="7" t="n"/>
-      <c r="E93" s="7" t="n"/>
+      <c r="A93" s="5" t="n"/>
+      <c r="B93" s="5" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="6" t="n"/>
     </row>
     <row r="94" ht="40" customHeight="1">
-      <c r="A94" s="6" t="n"/>
-      <c r="B94" s="6" t="n"/>
-      <c r="C94" s="7" t="n"/>
-      <c r="D94" s="7" t="n"/>
-      <c r="E94" s="7" t="n"/>
+      <c r="A94" s="5" t="n"/>
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="6" t="n"/>
     </row>
     <row r="95" ht="40" customHeight="1">
-      <c r="A95" s="6" t="n"/>
-      <c r="B95" s="6" t="n"/>
-      <c r="C95" s="7" t="n"/>
-      <c r="D95" s="7" t="n"/>
-      <c r="E95" s="7" t="n"/>
+      <c r="A95" s="5" t="n"/>
+      <c r="B95" s="5" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="6" t="n"/>
     </row>
     <row r="96" ht="40" customHeight="1">
-      <c r="A96" s="6" t="n"/>
-      <c r="B96" s="6" t="n"/>
-      <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="n"/>
-      <c r="E96" s="7" t="n"/>
+      <c r="A96" s="5" t="n"/>
+      <c r="B96" s="5" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
     </row>
     <row r="97" ht="40" customHeight="1">
-      <c r="A97" s="6" t="n"/>
-      <c r="B97" s="6" t="n"/>
-      <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
-      <c r="E97" s="7" t="n"/>
+      <c r="A97" s="5" t="n"/>
+      <c r="B97" s="5" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
     </row>
     <row r="98" ht="40" customHeight="1">
-      <c r="A98" s="6" t="n"/>
-      <c r="B98" s="6" t="n"/>
-      <c r="C98" s="7" t="n"/>
-      <c r="D98" s="7" t="n"/>
-      <c r="E98" s="7" t="n"/>
+      <c r="A98" s="5" t="n"/>
+      <c r="B98" s="5" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
     </row>
     <row r="99" ht="40" customHeight="1">
-      <c r="A99" s="6" t="n"/>
-      <c r="B99" s="6" t="n"/>
-      <c r="C99" s="7" t="n"/>
-      <c r="D99" s="7" t="n"/>
-      <c r="E99" s="7" t="n"/>
+      <c r="A99" s="5" t="n"/>
+      <c r="B99" s="5" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
     </row>
     <row r="100" ht="40" customHeight="1">
-      <c r="A100" s="6" t="n"/>
-      <c r="B100" s="6" t="n"/>
-      <c r="C100" s="7" t="n"/>
-      <c r="D100" s="7" t="n"/>
-      <c r="E100" s="7" t="n"/>
+      <c r="A100" s="5" t="n"/>
+      <c r="B100" s="5" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
     </row>
     <row r="101" ht="40" customHeight="1">
-      <c r="A101" s="6" t="n"/>
-      <c r="B101" s="6" t="n"/>
-      <c r="C101" s="7" t="n"/>
-      <c r="D101" s="7" t="n"/>
-      <c r="E101" s="7" t="n"/>
+      <c r="A101" s="5" t="n"/>
+      <c r="B101" s="5" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9139,7 +9138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9154,7 +9153,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>RESUMO ANUAL — 1º ANO</t>
         </is>
@@ -9212,27 +9211,27 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <f>Turma!B3</f>
+        <f>Turma!B2</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>IFERROR(('Presença - Fev'!AK3+'Presença - Mar'!AK3+'Presença - Abr'!AK3+'Presença - Mai'!AK3+'Presença - Jun'!AK3+'Presença - Jul'!AK3+'Presença - Ago'!AK3+'Presença - Set'!AK3+'Presença - Out'!AK3+'Presença - Nov'!AK3)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK2+'Presença - Mar'!AK2+'Presença - Abr'!AK2+'Presença - Mai'!AK2+'Presença - Jun'!AK2+'Presença - Jul'!AK2+'Presença - Ago'!AK2+'Presença - Set'!AK2+'Presença - Out'!AK2+'Presença - Nov'!AK2)/10,"")</f>
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'Notas - B1'!I3</f>
+        <f>'Notas - B1'!I2</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'Notas - B2'!I3</f>
+        <f>'Notas - B2'!I2</f>
         <v/>
       </c>
       <c r="F3" s="4">
-        <f>'Notas - B3'!I3</f>
+        <f>'Notas - B3'!I2</f>
         <v/>
       </c>
       <c r="G3" s="4">
-        <f>'Notas - B4'!I3</f>
+        <f>'Notas - B4'!I2</f>
         <v/>
       </c>
       <c r="H3" s="4">
@@ -9249,27 +9248,27 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <f>Turma!B4</f>
+        <f>Turma!B3</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>IFERROR(('Presença - Fev'!AK4+'Presença - Mar'!AK4+'Presença - Abr'!AK4+'Presença - Mai'!AK4+'Presença - Jun'!AK4+'Presença - Jul'!AK4+'Presença - Ago'!AK4+'Presença - Set'!AK4+'Presença - Out'!AK4+'Presença - Nov'!AK4)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK3+'Presença - Mar'!AK3+'Presença - Abr'!AK3+'Presença - Mai'!AK3+'Presença - Jun'!AK3+'Presença - Jul'!AK3+'Presença - Ago'!AK3+'Presença - Set'!AK3+'Presença - Out'!AK3+'Presença - Nov'!AK3)/10,"")</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'Notas - B1'!I4</f>
+        <f>'Notas - B1'!I3</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'Notas - B2'!I4</f>
+        <f>'Notas - B2'!I3</f>
         <v/>
       </c>
       <c r="F4" s="4">
-        <f>'Notas - B3'!I4</f>
+        <f>'Notas - B3'!I3</f>
         <v/>
       </c>
       <c r="G4" s="4">
-        <f>'Notas - B4'!I4</f>
+        <f>'Notas - B4'!I3</f>
         <v/>
       </c>
       <c r="H4" s="4">
@@ -9286,27 +9285,27 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <f>Turma!B5</f>
+        <f>Turma!B4</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>IFERROR(('Presença - Fev'!AK5+'Presença - Mar'!AK5+'Presença - Abr'!AK5+'Presença - Mai'!AK5+'Presença - Jun'!AK5+'Presença - Jul'!AK5+'Presença - Ago'!AK5+'Presença - Set'!AK5+'Presença - Out'!AK5+'Presença - Nov'!AK5)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK4+'Presença - Mar'!AK4+'Presença - Abr'!AK4+'Presença - Mai'!AK4+'Presença - Jun'!AK4+'Presença - Jul'!AK4+'Presença - Ago'!AK4+'Presença - Set'!AK4+'Presença - Out'!AK4+'Presença - Nov'!AK4)/10,"")</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'Notas - B1'!I5</f>
+        <f>'Notas - B1'!I4</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'Notas - B2'!I5</f>
+        <f>'Notas - B2'!I4</f>
         <v/>
       </c>
       <c r="F5" s="4">
-        <f>'Notas - B3'!I5</f>
+        <f>'Notas - B3'!I4</f>
         <v/>
       </c>
       <c r="G5" s="4">
-        <f>'Notas - B4'!I5</f>
+        <f>'Notas - B4'!I4</f>
         <v/>
       </c>
       <c r="H5" s="4">
@@ -9323,27 +9322,27 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <f>Turma!B6</f>
+        <f>Turma!B5</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>IFERROR(('Presença - Fev'!AK6+'Presença - Mar'!AK6+'Presença - Abr'!AK6+'Presença - Mai'!AK6+'Presença - Jun'!AK6+'Presença - Jul'!AK6+'Presença - Ago'!AK6+'Presença - Set'!AK6+'Presença - Out'!AK6+'Presença - Nov'!AK6)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK5+'Presença - Mar'!AK5+'Presença - Abr'!AK5+'Presença - Mai'!AK5+'Presença - Jun'!AK5+'Presença - Jul'!AK5+'Presença - Ago'!AK5+'Presença - Set'!AK5+'Presença - Out'!AK5+'Presença - Nov'!AK5)/10,"")</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>'Notas - B1'!I6</f>
+        <f>'Notas - B1'!I5</f>
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>'Notas - B2'!I6</f>
+        <f>'Notas - B2'!I5</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>'Notas - B3'!I6</f>
+        <f>'Notas - B3'!I5</f>
         <v/>
       </c>
       <c r="G6" s="4">
-        <f>'Notas - B4'!I6</f>
+        <f>'Notas - B4'!I5</f>
         <v/>
       </c>
       <c r="H6" s="4">
@@ -9360,27 +9359,27 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <f>Turma!B7</f>
+        <f>Turma!B6</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>IFERROR(('Presença - Fev'!AK7+'Presença - Mar'!AK7+'Presença - Abr'!AK7+'Presença - Mai'!AK7+'Presença - Jun'!AK7+'Presença - Jul'!AK7+'Presença - Ago'!AK7+'Presença - Set'!AK7+'Presença - Out'!AK7+'Presença - Nov'!AK7)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK6+'Presença - Mar'!AK6+'Presença - Abr'!AK6+'Presença - Mai'!AK6+'Presença - Jun'!AK6+'Presença - Jul'!AK6+'Presença - Ago'!AK6+'Presença - Set'!AK6+'Presença - Out'!AK6+'Presença - Nov'!AK6)/10,"")</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>'Notas - B1'!I7</f>
+        <f>'Notas - B1'!I6</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>'Notas - B2'!I7</f>
+        <f>'Notas - B2'!I6</f>
         <v/>
       </c>
       <c r="F7" s="4">
-        <f>'Notas - B3'!I7</f>
+        <f>'Notas - B3'!I6</f>
         <v/>
       </c>
       <c r="G7" s="4">
-        <f>'Notas - B4'!I7</f>
+        <f>'Notas - B4'!I6</f>
         <v/>
       </c>
       <c r="H7" s="4">
@@ -9397,27 +9396,27 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <f>Turma!B8</f>
+        <f>Turma!B7</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>IFERROR(('Presença - Fev'!AK8+'Presença - Mar'!AK8+'Presença - Abr'!AK8+'Presença - Mai'!AK8+'Presença - Jun'!AK8+'Presença - Jul'!AK8+'Presença - Ago'!AK8+'Presença - Set'!AK8+'Presença - Out'!AK8+'Presença - Nov'!AK8)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK7+'Presença - Mar'!AK7+'Presença - Abr'!AK7+'Presença - Mai'!AK7+'Presença - Jun'!AK7+'Presença - Jul'!AK7+'Presença - Ago'!AK7+'Presença - Set'!AK7+'Presença - Out'!AK7+'Presença - Nov'!AK7)/10,"")</f>
         <v/>
       </c>
       <c r="D8" s="4">
-        <f>'Notas - B1'!I8</f>
+        <f>'Notas - B1'!I7</f>
         <v/>
       </c>
       <c r="E8" s="4">
-        <f>'Notas - B2'!I8</f>
+        <f>'Notas - B2'!I7</f>
         <v/>
       </c>
       <c r="F8" s="4">
-        <f>'Notas - B3'!I8</f>
+        <f>'Notas - B3'!I7</f>
         <v/>
       </c>
       <c r="G8" s="4">
-        <f>'Notas - B4'!I8</f>
+        <f>'Notas - B4'!I7</f>
         <v/>
       </c>
       <c r="H8" s="4">
@@ -9434,27 +9433,27 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <f>Turma!B9</f>
+        <f>Turma!B8</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>IFERROR(('Presença - Fev'!AK9+'Presença - Mar'!AK9+'Presença - Abr'!AK9+'Presença - Mai'!AK9+'Presença - Jun'!AK9+'Presença - Jul'!AK9+'Presença - Ago'!AK9+'Presença - Set'!AK9+'Presença - Out'!AK9+'Presença - Nov'!AK9)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK8+'Presença - Mar'!AK8+'Presença - Abr'!AK8+'Presença - Mai'!AK8+'Presença - Jun'!AK8+'Presença - Jul'!AK8+'Presença - Ago'!AK8+'Presença - Set'!AK8+'Presença - Out'!AK8+'Presença - Nov'!AK8)/10,"")</f>
         <v/>
       </c>
       <c r="D9" s="4">
-        <f>'Notas - B1'!I9</f>
+        <f>'Notas - B1'!I8</f>
         <v/>
       </c>
       <c r="E9" s="4">
-        <f>'Notas - B2'!I9</f>
+        <f>'Notas - B2'!I8</f>
         <v/>
       </c>
       <c r="F9" s="4">
-        <f>'Notas - B3'!I9</f>
+        <f>'Notas - B3'!I8</f>
         <v/>
       </c>
       <c r="G9" s="4">
-        <f>'Notas - B4'!I9</f>
+        <f>'Notas - B4'!I8</f>
         <v/>
       </c>
       <c r="H9" s="4">
@@ -9471,27 +9470,27 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <f>Turma!B10</f>
+        <f>Turma!B9</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>IFERROR(('Presença - Fev'!AK10+'Presença - Mar'!AK10+'Presença - Abr'!AK10+'Presença - Mai'!AK10+'Presença - Jun'!AK10+'Presença - Jul'!AK10+'Presença - Ago'!AK10+'Presença - Set'!AK10+'Presença - Out'!AK10+'Presença - Nov'!AK10)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK9+'Presença - Mar'!AK9+'Presença - Abr'!AK9+'Presença - Mai'!AK9+'Presença - Jun'!AK9+'Presença - Jul'!AK9+'Presença - Ago'!AK9+'Presença - Set'!AK9+'Presença - Out'!AK9+'Presença - Nov'!AK9)/10,"")</f>
         <v/>
       </c>
       <c r="D10" s="4">
-        <f>'Notas - B1'!I10</f>
+        <f>'Notas - B1'!I9</f>
         <v/>
       </c>
       <c r="E10" s="4">
-        <f>'Notas - B2'!I10</f>
+        <f>'Notas - B2'!I9</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>'Notas - B3'!I10</f>
+        <f>'Notas - B3'!I9</f>
         <v/>
       </c>
       <c r="G10" s="4">
-        <f>'Notas - B4'!I10</f>
+        <f>'Notas - B4'!I9</f>
         <v/>
       </c>
       <c r="H10" s="4">
@@ -9508,27 +9507,27 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <f>Turma!B11</f>
+        <f>Turma!B10</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>IFERROR(('Presença - Fev'!AK11+'Presença - Mar'!AK11+'Presença - Abr'!AK11+'Presença - Mai'!AK11+'Presença - Jun'!AK11+'Presença - Jul'!AK11+'Presença - Ago'!AK11+'Presença - Set'!AK11+'Presença - Out'!AK11+'Presença - Nov'!AK11)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK10+'Presença - Mar'!AK10+'Presença - Abr'!AK10+'Presença - Mai'!AK10+'Presença - Jun'!AK10+'Presença - Jul'!AK10+'Presença - Ago'!AK10+'Presença - Set'!AK10+'Presença - Out'!AK10+'Presença - Nov'!AK10)/10,"")</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>'Notas - B1'!I11</f>
+        <f>'Notas - B1'!I10</f>
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>'Notas - B2'!I11</f>
+        <f>'Notas - B2'!I10</f>
         <v/>
       </c>
       <c r="F11" s="4">
-        <f>'Notas - B3'!I11</f>
+        <f>'Notas - B3'!I10</f>
         <v/>
       </c>
       <c r="G11" s="4">
-        <f>'Notas - B4'!I11</f>
+        <f>'Notas - B4'!I10</f>
         <v/>
       </c>
       <c r="H11" s="4">
@@ -9545,27 +9544,27 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <f>Turma!B12</f>
+        <f>Turma!B11</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>IFERROR(('Presença - Fev'!AK12+'Presença - Mar'!AK12+'Presença - Abr'!AK12+'Presença - Mai'!AK12+'Presença - Jun'!AK12+'Presença - Jul'!AK12+'Presença - Ago'!AK12+'Presença - Set'!AK12+'Presença - Out'!AK12+'Presença - Nov'!AK12)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK11+'Presença - Mar'!AK11+'Presença - Abr'!AK11+'Presença - Mai'!AK11+'Presença - Jun'!AK11+'Presença - Jul'!AK11+'Presença - Ago'!AK11+'Presença - Set'!AK11+'Presença - Out'!AK11+'Presença - Nov'!AK11)/10,"")</f>
         <v/>
       </c>
       <c r="D12" s="4">
-        <f>'Notas - B1'!I12</f>
+        <f>'Notas - B1'!I11</f>
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>'Notas - B2'!I12</f>
+        <f>'Notas - B2'!I11</f>
         <v/>
       </c>
       <c r="F12" s="4">
-        <f>'Notas - B3'!I12</f>
+        <f>'Notas - B3'!I11</f>
         <v/>
       </c>
       <c r="G12" s="4">
-        <f>'Notas - B4'!I12</f>
+        <f>'Notas - B4'!I11</f>
         <v/>
       </c>
       <c r="H12" s="4">
@@ -9582,27 +9581,27 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <f>Turma!B13</f>
+        <f>Turma!B12</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>IFERROR(('Presença - Fev'!AK13+'Presença - Mar'!AK13+'Presença - Abr'!AK13+'Presença - Mai'!AK13+'Presença - Jun'!AK13+'Presença - Jul'!AK13+'Presença - Ago'!AK13+'Presença - Set'!AK13+'Presença - Out'!AK13+'Presença - Nov'!AK13)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK12+'Presença - Mar'!AK12+'Presença - Abr'!AK12+'Presença - Mai'!AK12+'Presença - Jun'!AK12+'Presença - Jul'!AK12+'Presença - Ago'!AK12+'Presença - Set'!AK12+'Presença - Out'!AK12+'Presença - Nov'!AK12)/10,"")</f>
         <v/>
       </c>
       <c r="D13" s="4">
-        <f>'Notas - B1'!I13</f>
+        <f>'Notas - B1'!I12</f>
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>'Notas - B2'!I13</f>
+        <f>'Notas - B2'!I12</f>
         <v/>
       </c>
       <c r="F13" s="4">
-        <f>'Notas - B3'!I13</f>
+        <f>'Notas - B3'!I12</f>
         <v/>
       </c>
       <c r="G13" s="4">
-        <f>'Notas - B4'!I13</f>
+        <f>'Notas - B4'!I12</f>
         <v/>
       </c>
       <c r="H13" s="4">
@@ -9619,27 +9618,27 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <f>Turma!B14</f>
+        <f>Turma!B13</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>IFERROR(('Presença - Fev'!AK14+'Presença - Mar'!AK14+'Presença - Abr'!AK14+'Presença - Mai'!AK14+'Presença - Jun'!AK14+'Presença - Jul'!AK14+'Presença - Ago'!AK14+'Presença - Set'!AK14+'Presença - Out'!AK14+'Presença - Nov'!AK14)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK13+'Presença - Mar'!AK13+'Presença - Abr'!AK13+'Presença - Mai'!AK13+'Presença - Jun'!AK13+'Presença - Jul'!AK13+'Presença - Ago'!AK13+'Presença - Set'!AK13+'Presença - Out'!AK13+'Presença - Nov'!AK13)/10,"")</f>
         <v/>
       </c>
       <c r="D14" s="4">
-        <f>'Notas - B1'!I14</f>
+        <f>'Notas - B1'!I13</f>
         <v/>
       </c>
       <c r="E14" s="4">
-        <f>'Notas - B2'!I14</f>
+        <f>'Notas - B2'!I13</f>
         <v/>
       </c>
       <c r="F14" s="4">
-        <f>'Notas - B3'!I14</f>
+        <f>'Notas - B3'!I13</f>
         <v/>
       </c>
       <c r="G14" s="4">
-        <f>'Notas - B4'!I14</f>
+        <f>'Notas - B4'!I13</f>
         <v/>
       </c>
       <c r="H14" s="4">
@@ -9656,27 +9655,27 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <f>Turma!B15</f>
+        <f>Turma!B14</f>
         <v/>
       </c>
       <c r="C15" s="3">
-        <f>IFERROR(('Presença - Fev'!AK15+'Presença - Mar'!AK15+'Presença - Abr'!AK15+'Presença - Mai'!AK15+'Presença - Jun'!AK15+'Presença - Jul'!AK15+'Presença - Ago'!AK15+'Presença - Set'!AK15+'Presença - Out'!AK15+'Presença - Nov'!AK15)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK14+'Presença - Mar'!AK14+'Presença - Abr'!AK14+'Presença - Mai'!AK14+'Presença - Jun'!AK14+'Presença - Jul'!AK14+'Presença - Ago'!AK14+'Presença - Set'!AK14+'Presença - Out'!AK14+'Presença - Nov'!AK14)/10,"")</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>'Notas - B1'!I15</f>
+        <f>'Notas - B1'!I14</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>'Notas - B2'!I15</f>
+        <f>'Notas - B2'!I14</f>
         <v/>
       </c>
       <c r="F15" s="4">
-        <f>'Notas - B3'!I15</f>
+        <f>'Notas - B3'!I14</f>
         <v/>
       </c>
       <c r="G15" s="4">
-        <f>'Notas - B4'!I15</f>
+        <f>'Notas - B4'!I14</f>
         <v/>
       </c>
       <c r="H15" s="4">
@@ -9693,27 +9692,27 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <f>Turma!B16</f>
+        <f>Turma!B15</f>
         <v/>
       </c>
       <c r="C16" s="3">
-        <f>IFERROR(('Presença - Fev'!AK16+'Presença - Mar'!AK16+'Presença - Abr'!AK16+'Presença - Mai'!AK16+'Presença - Jun'!AK16+'Presença - Jul'!AK16+'Presença - Ago'!AK16+'Presença - Set'!AK16+'Presença - Out'!AK16+'Presença - Nov'!AK16)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK15+'Presença - Mar'!AK15+'Presença - Abr'!AK15+'Presença - Mai'!AK15+'Presença - Jun'!AK15+'Presença - Jul'!AK15+'Presença - Ago'!AK15+'Presença - Set'!AK15+'Presença - Out'!AK15+'Presença - Nov'!AK15)/10,"")</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>'Notas - B1'!I16</f>
+        <f>'Notas - B1'!I15</f>
         <v/>
       </c>
       <c r="E16" s="4">
-        <f>'Notas - B2'!I16</f>
+        <f>'Notas - B2'!I15</f>
         <v/>
       </c>
       <c r="F16" s="4">
-        <f>'Notas - B3'!I16</f>
+        <f>'Notas - B3'!I15</f>
         <v/>
       </c>
       <c r="G16" s="4">
-        <f>'Notas - B4'!I16</f>
+        <f>'Notas - B4'!I15</f>
         <v/>
       </c>
       <c r="H16" s="4">
@@ -9730,27 +9729,27 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <f>Turma!B17</f>
+        <f>Turma!B16</f>
         <v/>
       </c>
       <c r="C17" s="3">
-        <f>IFERROR(('Presença - Fev'!AK17+'Presença - Mar'!AK17+'Presença - Abr'!AK17+'Presença - Mai'!AK17+'Presença - Jun'!AK17+'Presença - Jul'!AK17+'Presença - Ago'!AK17+'Presença - Set'!AK17+'Presença - Out'!AK17+'Presença - Nov'!AK17)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK16+'Presença - Mar'!AK16+'Presença - Abr'!AK16+'Presença - Mai'!AK16+'Presença - Jun'!AK16+'Presença - Jul'!AK16+'Presença - Ago'!AK16+'Presença - Set'!AK16+'Presença - Out'!AK16+'Presença - Nov'!AK16)/10,"")</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>'Notas - B1'!I17</f>
+        <f>'Notas - B1'!I16</f>
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>'Notas - B2'!I17</f>
+        <f>'Notas - B2'!I16</f>
         <v/>
       </c>
       <c r="F17" s="4">
-        <f>'Notas - B3'!I17</f>
+        <f>'Notas - B3'!I16</f>
         <v/>
       </c>
       <c r="G17" s="4">
-        <f>'Notas - B4'!I17</f>
+        <f>'Notas - B4'!I16</f>
         <v/>
       </c>
       <c r="H17" s="4">
@@ -9767,27 +9766,27 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <f>Turma!B18</f>
+        <f>Turma!B17</f>
         <v/>
       </c>
       <c r="C18" s="3">
-        <f>IFERROR(('Presença - Fev'!AK18+'Presença - Mar'!AK18+'Presença - Abr'!AK18+'Presença - Mai'!AK18+'Presença - Jun'!AK18+'Presença - Jul'!AK18+'Presença - Ago'!AK18+'Presença - Set'!AK18+'Presença - Out'!AK18+'Presença - Nov'!AK18)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK17+'Presença - Mar'!AK17+'Presença - Abr'!AK17+'Presença - Mai'!AK17+'Presença - Jun'!AK17+'Presença - Jul'!AK17+'Presença - Ago'!AK17+'Presença - Set'!AK17+'Presença - Out'!AK17+'Presença - Nov'!AK17)/10,"")</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>'Notas - B1'!I18</f>
+        <f>'Notas - B1'!I17</f>
         <v/>
       </c>
       <c r="E18" s="4">
-        <f>'Notas - B2'!I18</f>
+        <f>'Notas - B2'!I17</f>
         <v/>
       </c>
       <c r="F18" s="4">
-        <f>'Notas - B3'!I18</f>
+        <f>'Notas - B3'!I17</f>
         <v/>
       </c>
       <c r="G18" s="4">
-        <f>'Notas - B4'!I18</f>
+        <f>'Notas - B4'!I17</f>
         <v/>
       </c>
       <c r="H18" s="4">
@@ -9804,27 +9803,27 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <f>Turma!B19</f>
+        <f>Turma!B18</f>
         <v/>
       </c>
       <c r="C19" s="3">
-        <f>IFERROR(('Presença - Fev'!AK19+'Presença - Mar'!AK19+'Presença - Abr'!AK19+'Presença - Mai'!AK19+'Presença - Jun'!AK19+'Presença - Jul'!AK19+'Presença - Ago'!AK19+'Presença - Set'!AK19+'Presença - Out'!AK19+'Presença - Nov'!AK19)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK18+'Presença - Mar'!AK18+'Presença - Abr'!AK18+'Presença - Mai'!AK18+'Presença - Jun'!AK18+'Presença - Jul'!AK18+'Presença - Ago'!AK18+'Presença - Set'!AK18+'Presença - Out'!AK18+'Presença - Nov'!AK18)/10,"")</f>
         <v/>
       </c>
       <c r="D19" s="4">
-        <f>'Notas - B1'!I19</f>
+        <f>'Notas - B1'!I18</f>
         <v/>
       </c>
       <c r="E19" s="4">
-        <f>'Notas - B2'!I19</f>
+        <f>'Notas - B2'!I18</f>
         <v/>
       </c>
       <c r="F19" s="4">
-        <f>'Notas - B3'!I19</f>
+        <f>'Notas - B3'!I18</f>
         <v/>
       </c>
       <c r="G19" s="4">
-        <f>'Notas - B4'!I19</f>
+        <f>'Notas - B4'!I18</f>
         <v/>
       </c>
       <c r="H19" s="4">
@@ -9841,27 +9840,27 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <f>Turma!B20</f>
+        <f>Turma!B19</f>
         <v/>
       </c>
       <c r="C20" s="3">
-        <f>IFERROR(('Presença - Fev'!AK20+'Presença - Mar'!AK20+'Presença - Abr'!AK20+'Presença - Mai'!AK20+'Presença - Jun'!AK20+'Presença - Jul'!AK20+'Presença - Ago'!AK20+'Presença - Set'!AK20+'Presença - Out'!AK20+'Presença - Nov'!AK20)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK19+'Presença - Mar'!AK19+'Presença - Abr'!AK19+'Presença - Mai'!AK19+'Presença - Jun'!AK19+'Presença - Jul'!AK19+'Presença - Ago'!AK19+'Presença - Set'!AK19+'Presença - Out'!AK19+'Presença - Nov'!AK19)/10,"")</f>
         <v/>
       </c>
       <c r="D20" s="4">
-        <f>'Notas - B1'!I20</f>
+        <f>'Notas - B1'!I19</f>
         <v/>
       </c>
       <c r="E20" s="4">
-        <f>'Notas - B2'!I20</f>
+        <f>'Notas - B2'!I19</f>
         <v/>
       </c>
       <c r="F20" s="4">
-        <f>'Notas - B3'!I20</f>
+        <f>'Notas - B3'!I19</f>
         <v/>
       </c>
       <c r="G20" s="4">
-        <f>'Notas - B4'!I20</f>
+        <f>'Notas - B4'!I19</f>
         <v/>
       </c>
       <c r="H20" s="4">
@@ -9878,27 +9877,27 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <f>Turma!B21</f>
+        <f>Turma!B20</f>
         <v/>
       </c>
       <c r="C21" s="3">
-        <f>IFERROR(('Presença - Fev'!AK21+'Presença - Mar'!AK21+'Presença - Abr'!AK21+'Presença - Mai'!AK21+'Presença - Jun'!AK21+'Presença - Jul'!AK21+'Presença - Ago'!AK21+'Presença - Set'!AK21+'Presença - Out'!AK21+'Presença - Nov'!AK21)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK20+'Presença - Mar'!AK20+'Presença - Abr'!AK20+'Presença - Mai'!AK20+'Presença - Jun'!AK20+'Presença - Jul'!AK20+'Presença - Ago'!AK20+'Presença - Set'!AK20+'Presença - Out'!AK20+'Presença - Nov'!AK20)/10,"")</f>
         <v/>
       </c>
       <c r="D21" s="4">
-        <f>'Notas - B1'!I21</f>
+        <f>'Notas - B1'!I20</f>
         <v/>
       </c>
       <c r="E21" s="4">
-        <f>'Notas - B2'!I21</f>
+        <f>'Notas - B2'!I20</f>
         <v/>
       </c>
       <c r="F21" s="4">
-        <f>'Notas - B3'!I21</f>
+        <f>'Notas - B3'!I20</f>
         <v/>
       </c>
       <c r="G21" s="4">
-        <f>'Notas - B4'!I21</f>
+        <f>'Notas - B4'!I20</f>
         <v/>
       </c>
       <c r="H21" s="4">
@@ -9915,27 +9914,27 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <f>Turma!B22</f>
+        <f>Turma!B21</f>
         <v/>
       </c>
       <c r="C22" s="3">
-        <f>IFERROR(('Presença - Fev'!AK22+'Presença - Mar'!AK22+'Presença - Abr'!AK22+'Presença - Mai'!AK22+'Presença - Jun'!AK22+'Presença - Jul'!AK22+'Presença - Ago'!AK22+'Presença - Set'!AK22+'Presença - Out'!AK22+'Presença - Nov'!AK22)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK21+'Presença - Mar'!AK21+'Presença - Abr'!AK21+'Presença - Mai'!AK21+'Presença - Jun'!AK21+'Presença - Jul'!AK21+'Presença - Ago'!AK21+'Presença - Set'!AK21+'Presença - Out'!AK21+'Presença - Nov'!AK21)/10,"")</f>
         <v/>
       </c>
       <c r="D22" s="4">
-        <f>'Notas - B1'!I22</f>
+        <f>'Notas - B1'!I21</f>
         <v/>
       </c>
       <c r="E22" s="4">
-        <f>'Notas - B2'!I22</f>
+        <f>'Notas - B2'!I21</f>
         <v/>
       </c>
       <c r="F22" s="4">
-        <f>'Notas - B3'!I22</f>
+        <f>'Notas - B3'!I21</f>
         <v/>
       </c>
       <c r="G22" s="4">
-        <f>'Notas - B4'!I22</f>
+        <f>'Notas - B4'!I21</f>
         <v/>
       </c>
       <c r="H22" s="4">
@@ -9952,27 +9951,27 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <f>Turma!B23</f>
+        <f>Turma!B22</f>
         <v/>
       </c>
       <c r="C23" s="3">
-        <f>IFERROR(('Presença - Fev'!AK23+'Presença - Mar'!AK23+'Presença - Abr'!AK23+'Presença - Mai'!AK23+'Presença - Jun'!AK23+'Presença - Jul'!AK23+'Presença - Ago'!AK23+'Presença - Set'!AK23+'Presença - Out'!AK23+'Presença - Nov'!AK23)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK22+'Presença - Mar'!AK22+'Presença - Abr'!AK22+'Presença - Mai'!AK22+'Presença - Jun'!AK22+'Presença - Jul'!AK22+'Presença - Ago'!AK22+'Presença - Set'!AK22+'Presença - Out'!AK22+'Presença - Nov'!AK22)/10,"")</f>
         <v/>
       </c>
       <c r="D23" s="4">
-        <f>'Notas - B1'!I23</f>
+        <f>'Notas - B1'!I22</f>
         <v/>
       </c>
       <c r="E23" s="4">
-        <f>'Notas - B2'!I23</f>
+        <f>'Notas - B2'!I22</f>
         <v/>
       </c>
       <c r="F23" s="4">
-        <f>'Notas - B3'!I23</f>
+        <f>'Notas - B3'!I22</f>
         <v/>
       </c>
       <c r="G23" s="4">
-        <f>'Notas - B4'!I23</f>
+        <f>'Notas - B4'!I22</f>
         <v/>
       </c>
       <c r="H23" s="4">
@@ -9989,27 +9988,27 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <f>Turma!B24</f>
+        <f>Turma!B23</f>
         <v/>
       </c>
       <c r="C24" s="3">
-        <f>IFERROR(('Presença - Fev'!AK24+'Presença - Mar'!AK24+'Presença - Abr'!AK24+'Presença - Mai'!AK24+'Presença - Jun'!AK24+'Presença - Jul'!AK24+'Presença - Ago'!AK24+'Presença - Set'!AK24+'Presença - Out'!AK24+'Presença - Nov'!AK24)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK23+'Presença - Mar'!AK23+'Presença - Abr'!AK23+'Presença - Mai'!AK23+'Presença - Jun'!AK23+'Presença - Jul'!AK23+'Presença - Ago'!AK23+'Presença - Set'!AK23+'Presença - Out'!AK23+'Presença - Nov'!AK23)/10,"")</f>
         <v/>
       </c>
       <c r="D24" s="4">
-        <f>'Notas - B1'!I24</f>
+        <f>'Notas - B1'!I23</f>
         <v/>
       </c>
       <c r="E24" s="4">
-        <f>'Notas - B2'!I24</f>
+        <f>'Notas - B2'!I23</f>
         <v/>
       </c>
       <c r="F24" s="4">
-        <f>'Notas - B3'!I24</f>
+        <f>'Notas - B3'!I23</f>
         <v/>
       </c>
       <c r="G24" s="4">
-        <f>'Notas - B4'!I24</f>
+        <f>'Notas - B4'!I23</f>
         <v/>
       </c>
       <c r="H24" s="4">
@@ -10026,27 +10025,27 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <f>Turma!B25</f>
+        <f>Turma!B24</f>
         <v/>
       </c>
       <c r="C25" s="3">
-        <f>IFERROR(('Presença - Fev'!AK25+'Presença - Mar'!AK25+'Presença - Abr'!AK25+'Presença - Mai'!AK25+'Presença - Jun'!AK25+'Presença - Jul'!AK25+'Presença - Ago'!AK25+'Presença - Set'!AK25+'Presença - Out'!AK25+'Presença - Nov'!AK25)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK24+'Presença - Mar'!AK24+'Presença - Abr'!AK24+'Presença - Mai'!AK24+'Presença - Jun'!AK24+'Presença - Jul'!AK24+'Presença - Ago'!AK24+'Presença - Set'!AK24+'Presença - Out'!AK24+'Presença - Nov'!AK24)/10,"")</f>
         <v/>
       </c>
       <c r="D25" s="4">
-        <f>'Notas - B1'!I25</f>
+        <f>'Notas - B1'!I24</f>
         <v/>
       </c>
       <c r="E25" s="4">
-        <f>'Notas - B2'!I25</f>
+        <f>'Notas - B2'!I24</f>
         <v/>
       </c>
       <c r="F25" s="4">
-        <f>'Notas - B3'!I25</f>
+        <f>'Notas - B3'!I24</f>
         <v/>
       </c>
       <c r="G25" s="4">
-        <f>'Notas - B4'!I25</f>
+        <f>'Notas - B4'!I24</f>
         <v/>
       </c>
       <c r="H25" s="4">
@@ -10063,27 +10062,27 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <f>Turma!B26</f>
+        <f>Turma!B25</f>
         <v/>
       </c>
       <c r="C26" s="3">
-        <f>IFERROR(('Presença - Fev'!AK26+'Presença - Mar'!AK26+'Presença - Abr'!AK26+'Presença - Mai'!AK26+'Presença - Jun'!AK26+'Presença - Jul'!AK26+'Presença - Ago'!AK26+'Presença - Set'!AK26+'Presença - Out'!AK26+'Presença - Nov'!AK26)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK25+'Presença - Mar'!AK25+'Presença - Abr'!AK25+'Presença - Mai'!AK25+'Presença - Jun'!AK25+'Presença - Jul'!AK25+'Presença - Ago'!AK25+'Presença - Set'!AK25+'Presença - Out'!AK25+'Presença - Nov'!AK25)/10,"")</f>
         <v/>
       </c>
       <c r="D26" s="4">
-        <f>'Notas - B1'!I26</f>
+        <f>'Notas - B1'!I25</f>
         <v/>
       </c>
       <c r="E26" s="4">
-        <f>'Notas - B2'!I26</f>
+        <f>'Notas - B2'!I25</f>
         <v/>
       </c>
       <c r="F26" s="4">
-        <f>'Notas - B3'!I26</f>
+        <f>'Notas - B3'!I25</f>
         <v/>
       </c>
       <c r="G26" s="4">
-        <f>'Notas - B4'!I26</f>
+        <f>'Notas - B4'!I25</f>
         <v/>
       </c>
       <c r="H26" s="4">
@@ -10100,27 +10099,27 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <f>Turma!B27</f>
+        <f>Turma!B26</f>
         <v/>
       </c>
       <c r="C27" s="3">
-        <f>IFERROR(('Presença - Fev'!AK27+'Presença - Mar'!AK27+'Presença - Abr'!AK27+'Presença - Mai'!AK27+'Presença - Jun'!AK27+'Presença - Jul'!AK27+'Presença - Ago'!AK27+'Presença - Set'!AK27+'Presença - Out'!AK27+'Presença - Nov'!AK27)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK26+'Presença - Mar'!AK26+'Presença - Abr'!AK26+'Presença - Mai'!AK26+'Presença - Jun'!AK26+'Presença - Jul'!AK26+'Presença - Ago'!AK26+'Presença - Set'!AK26+'Presença - Out'!AK26+'Presença - Nov'!AK26)/10,"")</f>
         <v/>
       </c>
       <c r="D27" s="4">
-        <f>'Notas - B1'!I27</f>
+        <f>'Notas - B1'!I26</f>
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>'Notas - B2'!I27</f>
+        <f>'Notas - B2'!I26</f>
         <v/>
       </c>
       <c r="F27" s="4">
-        <f>'Notas - B3'!I27</f>
+        <f>'Notas - B3'!I26</f>
         <v/>
       </c>
       <c r="G27" s="4">
-        <f>'Notas - B4'!I27</f>
+        <f>'Notas - B4'!I26</f>
         <v/>
       </c>
       <c r="H27" s="4">
@@ -10137,27 +10136,27 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <f>Turma!B28</f>
+        <f>Turma!B27</f>
         <v/>
       </c>
       <c r="C28" s="3">
-        <f>IFERROR(('Presença - Fev'!AK28+'Presença - Mar'!AK28+'Presença - Abr'!AK28+'Presença - Mai'!AK28+'Presença - Jun'!AK28+'Presença - Jul'!AK28+'Presença - Ago'!AK28+'Presença - Set'!AK28+'Presença - Out'!AK28+'Presença - Nov'!AK28)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK27+'Presença - Mar'!AK27+'Presença - Abr'!AK27+'Presença - Mai'!AK27+'Presença - Jun'!AK27+'Presença - Jul'!AK27+'Presença - Ago'!AK27+'Presença - Set'!AK27+'Presença - Out'!AK27+'Presença - Nov'!AK27)/10,"")</f>
         <v/>
       </c>
       <c r="D28" s="4">
-        <f>'Notas - B1'!I28</f>
+        <f>'Notas - B1'!I27</f>
         <v/>
       </c>
       <c r="E28" s="4">
-        <f>'Notas - B2'!I28</f>
+        <f>'Notas - B2'!I27</f>
         <v/>
       </c>
       <c r="F28" s="4">
-        <f>'Notas - B3'!I28</f>
+        <f>'Notas - B3'!I27</f>
         <v/>
       </c>
       <c r="G28" s="4">
-        <f>'Notas - B4'!I28</f>
+        <f>'Notas - B4'!I27</f>
         <v/>
       </c>
       <c r="H28" s="4">
@@ -10174,27 +10173,27 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <f>Turma!B29</f>
+        <f>Turma!B28</f>
         <v/>
       </c>
       <c r="C29" s="3">
-        <f>IFERROR(('Presença - Fev'!AK29+'Presença - Mar'!AK29+'Presença - Abr'!AK29+'Presença - Mai'!AK29+'Presença - Jun'!AK29+'Presença - Jul'!AK29+'Presença - Ago'!AK29+'Presença - Set'!AK29+'Presença - Out'!AK29+'Presença - Nov'!AK29)/10,"")</f>
+        <f>IFERROR(('Presença - Fev'!AK28+'Presença - Mar'!AK28+'Presença - Abr'!AK28+'Presença - Mai'!AK28+'Presença - Jun'!AK28+'Presença - Jul'!AK28+'Presença - Ago'!AK28+'Presença - Set'!AK28+'Presença - Out'!AK28+'Presença - Nov'!AK28)/10,"")</f>
         <v/>
       </c>
       <c r="D29" s="4">
-        <f>'Notas - B1'!I29</f>
+        <f>'Notas - B1'!I28</f>
         <v/>
       </c>
       <c r="E29" s="4">
-        <f>'Notas - B2'!I29</f>
+        <f>'Notas - B2'!I28</f>
         <v/>
       </c>
       <c r="F29" s="4">
-        <f>'Notas - B3'!I29</f>
+        <f>'Notas - B3'!I28</f>
         <v/>
       </c>
       <c r="G29" s="4">
-        <f>'Notas - B4'!I29</f>
+        <f>'Notas - B4'!I28</f>
         <v/>
       </c>
       <c r="H29" s="4">
@@ -10208,7 +10207,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I29">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">

</xml_diff>

<commit_message>
feat: cores de nota azul/vermelho, .gitignore e README
</commit_message>
<xml_diff>
--- a/diario-de-classe.xlsx
+++ b/diario-de-classe.xlsx
@@ -131,14 +131,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFEB9C"/>
+          <fgColor rgb="00DDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
+          <fgColor rgb="00FFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5066,12 +5066,8 @@
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
       <formula>5</formula>
-      <formula>6.99</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
-      <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5664,12 +5660,8 @@
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
       <formula>5</formula>
-      <formula>6.99</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
-      <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6262,12 +6254,8 @@
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
       <formula>5</formula>
-      <formula>6.99</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
-      <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6860,12 +6848,8 @@
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
       <formula>5</formula>
-      <formula>6.99</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="2">
-      <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7410,7 +7394,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G41">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Aprovado"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
@@ -10210,13 +10194,13 @@
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I29">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Aprovado"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"Recuperação"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Rec. Freq."</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>